<commit_message>
Fix: Zero TDS sheet uses actual section per entry, not hardcoded 194C
- Collect below-threshold entries from ALL sections via unmatched_tally dict
- Tag each entry with _section from its section key
- Group by (vendor, section) instead of just vendor
- Use section-specific threshold descriptions (₹1L for 194C, ₹30K for 194J, etc.)
- Backward compatible with old unmatched_tally_194c/194a keys

https://claude.ai/code/session_01U1MuRvDgn4XPQ38Fe5qjWF
</commit_message>
<xml_diff>
--- a/tds-recon/data/results/tds_recon_report.xlsx
+++ b/tds-recon/data/results/tds_recon_report.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Issues for Review" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="TDS Report - Matched" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Zero TDS - Exempt" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issues for Review" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TDS Report - Matched" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zero TDS - Exempt" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Issues for Review'!$A$1:$J$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'TDS Report - Matched'!$A$1:$Q$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Issues for Review'!$A$1:$J$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'TDS Report - Matched'!$A$1:$Q$80</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Zero TDS - Exempt'!$A$1:$G$68</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -546,31 +546,31 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>missing_tds</t>
+          <t>partial_tds</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Kamal Kishor Bagri</t>
+          <t>Sahib S Choudhary &amp; Co.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>194H</t>
+          <t>194J(b)</t>
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>16845</v>
+        <v>30000</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>No Form 26 entry found for Kamal Kishor Bagri under 194H. Tally shows ₹16,845 in Brokerage and Commission, Brokerage and Commission_18%. TDS may be missing.</t>
+          <t>Vendor Sahib S Choudhary &amp; Co. has Form 26 entry under 194J(b) but additional ₹30,000 in books (Audit Fees) is not covered. TDS may be short-deducted.</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Tally shows expenses to this vendor but no TDS was deducted in Form 26. Action required: (1) Check if vendor provided Form 15G/15H or lower deduction certificate. (2) If not, deduct TDS immediately and deposit with interest u/s 201(1A) at 1% per month. (3) File revised TDS return for the applicable quarter.</t>
+          <t>Manual review required.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -580,88 +580,92 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>missing_tds</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Kochar Tradelink LLP</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>194H</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>83675</v>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>No Form 26 entry found for Kochar Tradelink LLP under 194H. Tally shows ₹83,675 in Brokerage and Commission, Brokerage and Commission_18%. TDS may be missing.</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Tally shows expenses to this vendor but no TDS was deducted in Form 26. Action required: (1) Check if vendor provided Form 15G/15H or lower deduction certificate. (2) If not, deduct TDS immediately and deposit with interest u/s 201(1A) at 1% per month. (3) File revised TDS return for the applicable quarter.</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>section_validation</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ANDREAL INNOVATION PVT LTD</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>ABACA2255R</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>194C</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Ambiguous expense(s): Advertisement. Section 194C is possible but verify against invoice/contract nature.</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Ambiguous classification — verify invoice nature. If advertisement is creative/professional service → 194J(b). If it's production/printing contract work → 194C. Obtain vendor declaration if uncertain.</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>missing_tds</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Pukesh Sharma</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>194H</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>20877</v>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>No Form 26 entry found for Pukesh Sharma under 194H. Tally shows ₹20,877 in Brokerage and Commission. TDS may be missing.</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Tally shows expenses to this vendor but no TDS was deducted in Form 26. Action required: (1) Check if vendor provided Form 15G/15H or lower deduction certificate. (2) If not, deduct TDS immediately and deposit with interest u/s 201(1A) at 1% per month. (3) File revised TDS return for the applicable quarter.</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>section_validation</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>ANDERSON TECHNOLOGY PVT LTD</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>AAFCA4805K</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>194C</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr"/>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Ambiguous expense(s): Advertisement. Section 194C is possible but verify against invoice/contract nature.</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Ambiguous classification — verify invoice nature. If advertisement is creative/professional service → 194J(b). If it's production/printing contract work → 194C. Obtain vendor declaration if uncertain.</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -683,12 +687,12 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>ANDREAL INNOVATION PVT LTD</t>
+          <t>ANDERSON TECHNOLOGY PVT LTD</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>ABACA2255R</t>
+          <t>AAFCA4805K</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -775,12 +779,12 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>ANDERSON TECHNOLOGY PVT LTD</t>
+          <t>ANDREAL INNOVATION PVT LTD</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>AAFCA4805K</t>
+          <t>ABACA2255R</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -816,33 +820,31 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>section_validation</t>
+          <t>missing_tds</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>ANDERSON TECHNOLOGY PVT LTD</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>AAFCA4805K</t>
-        </is>
-      </c>
+          <t>Kochar Tradelink LLP</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>194C</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr"/>
+          <t>194H</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>44932</v>
+      </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Ambiguous expense(s): Advertisement. Section 194C is possible but verify against invoice/contract nature.</t>
+          <t>No Form 26 entry found for Kochar Tradelink LLP under 194H. Tally shows ₹44,932 in Brokerage and Commission. TDS may be missing. Review: Has entries on quarter/year-end dates (2025-03-31) alongside other dates — may include provisions or reversals. | Same transaction (₹38,743) appears in both Journal Register and GST Exp Register — counted once from Journal. Please confirm these are the same entry.</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Ambiguous classification — verify invoice nature. If advertisement is creative/professional service → 194J(b). If it's production/printing contract work → 194C. Obtain vendor declaration if uncertain.</t>
+          <t>Tally shows expenses to this vendor but no TDS was deducted in Form 26. Action required: (1) Check if vendor provided Form 15G/15H or lower deduction certificate. (2) If not, deduct TDS immediately and deposit with interest u/s 201(1A) at 1% per month. (3) File revised TDS return for the applicable quarter.</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
@@ -862,43 +864,231 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
+          <t>missing_tds</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Pukesh Sharma</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>194H</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>20877</v>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>No Form 26 entry found for Pukesh Sharma under 194H. Tally shows ₹20,877 in Brokerage and Commission. TDS may be missing. Review: Has entries on quarter/year-end dates (2025-03-31) alongside other dates — may include provisions or reversals.</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Tally shows expenses to this vendor but no TDS was deducted in Form 26. Action required: (1) Check if vendor provided Form 15G/15H or lower deduction certificate. (2) If not, deduct TDS immediately and deposit with interest u/s 201(1A) at 1% per month. (3) File revised TDS return for the applicable quarter.</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
           <t>section_validation</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>ANDREAL INNOVATION PVT LTD</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>ABACA2255R</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>194C</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr"/>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>Ambiguous expense(s): Advertisement. Section 194C is possible but verify against invoice/contract nature.</t>
-        </is>
-      </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>Ambiguous classification — verify invoice nature. If advertisement is creative/professional service → 194J(b). If it's production/printing contract work → 194C. Obtain vendor declaration if uncertain.</t>
-        </is>
-      </c>
-      <c r="J9" s="3" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>GST PROFESSIONALS LLP</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>AAPFG3370E</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>194J(b)</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr"/>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Cannot classify expense(s): Professonal Charges. Manual review needed.</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>Expense head could not be auto-classified. Manually review the vendor invoice and assign the correct TDS section.</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>threshold_validation</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>SAHIB S CHOUDHARY &amp; COMPANY</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>AEJPC0634D</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>194J(b)</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>9000</v>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>194J(b) for SAHIB S CHOUDHARY &amp; COMPANY: aggregate ₹9,000 is below annual threshold ₹30,000. TDS deduction is not mandatory (but not wrong if deducted).</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>TDS was deducted even though aggregate amount is below the threshold. This is not an error — voluntary TDS deduction is valid. No action needed, but note for internal records.</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>threshold_validation</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Raymond Limited</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>AAACR4896A</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>194Q</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>1480982</v>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>194Q for Raymond Limited: aggregate ₹1,480,982 is below annual threshold ₹5,000,000. TDS deduction is not mandatory (but not wrong if deducted).</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>TDS was deducted even though aggregate amount is below the threshold. This is not an error — voluntary TDS deduction is valid. No action needed, but note for internal records.</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>threshold_validation</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Sai Boutique</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>AEPFS3230M</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>194Q</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>381820</v>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>194Q for Sai Boutique: aggregate ₹381,820 is below annual threshold ₹5,000,000. TDS deduction is not mandatory (but not wrong if deducted).</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>TDS was deducted even though aggregate amount is below the threshold. This is not an error — voluntary TDS deduction is valid. No action needed, but note for internal records.</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J9"/>
+  <autoFilter ref="A1:J13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -909,7 +1099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q57"/>
+  <dimension ref="A1:Q80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4994,8 +5184,1613 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="4" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Amar Nath Prasad</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>BNAPP1451L</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>194H</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="n">
+        <v>22090</v>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="G58" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H58" s="4" t="n">
+        <v>442</v>
+      </c>
+      <c r="I58" s="4" t="inlineStr">
+        <is>
+          <t>Amar Nath Prasad Harsh Dudheria</t>
+        </is>
+      </c>
+      <c r="J58" s="4" t="n">
+        <v>22090</v>
+      </c>
+      <c r="K58" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="L58" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M58" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N58" s="4" t="inlineStr">
+        <is>
+          <t>fuzzy_match</t>
+        </is>
+      </c>
+      <c r="O58" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P58" s="4" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="Q58" s="4" t="inlineStr">
+        <is>
+          <t>Brokerage and Commission</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>Ankit Poddar</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>BFIPP7592G</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>194H</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="n">
+        <v>68301</v>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="G59" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H59" s="4" t="n">
+        <v>1366</v>
+      </c>
+      <c r="I59" s="4" t="inlineStr">
+        <is>
+          <t>Ankit Poddar</t>
+        </is>
+      </c>
+      <c r="J59" s="4" t="n">
+        <v>68301</v>
+      </c>
+      <c r="K59" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="L59" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M59" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N59" s="4" t="inlineStr">
+        <is>
+          <t>exact_match</t>
+        </is>
+      </c>
+      <c r="O59" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P59" s="4" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="Q59" s="4" t="inlineStr">
+        <is>
+          <t>Brokerage and Commission</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>Ankit Sadani</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>JBNPS5946C</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>194H</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="n">
+        <v>267137</v>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="G60" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H60" s="4" t="n">
+        <v>5343</v>
+      </c>
+      <c r="I60" s="4" t="inlineStr">
+        <is>
+          <t>Ankit Sadani</t>
+        </is>
+      </c>
+      <c r="J60" s="4" t="n">
+        <v>267137</v>
+      </c>
+      <c r="K60" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="L60" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M60" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N60" s="4" t="inlineStr">
+        <is>
+          <t>exact_match</t>
+        </is>
+      </c>
+      <c r="O60" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P60" s="4" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="Q60" s="4" t="inlineStr">
+        <is>
+          <t>Brokerage and Commission</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>Dhirendra Lalitray Doshi</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>AEXPD1479B</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>194H</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="n">
+        <v>55200</v>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H61" s="4" t="n">
+        <v>1104</v>
+      </c>
+      <c r="I61" s="4" t="inlineStr">
+        <is>
+          <t>Dhirendra Lalitray Doshi</t>
+        </is>
+      </c>
+      <c r="J61" s="4" t="n">
+        <v>55200</v>
+      </c>
+      <c r="K61" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="L61" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M61" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N61" s="4" t="inlineStr">
+        <is>
+          <t>exact_match</t>
+        </is>
+      </c>
+      <c r="O61" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P61" s="4" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="Q61" s="4" t="inlineStr">
+        <is>
+          <t>Brokerage and Commission</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>HASMUKH VITHALDAS JOISHER</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>ADNPJ5114E</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>194H</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="n">
+        <v>111532</v>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H62" s="4" t="n">
+        <v>2231</v>
+      </c>
+      <c r="I62" s="4" t="inlineStr">
+        <is>
+          <t>Hasmukh Vithaldas Joisher</t>
+        </is>
+      </c>
+      <c r="J62" s="4" t="n">
+        <v>111532</v>
+      </c>
+      <c r="K62" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="L62" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M62" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N62" s="4" t="inlineStr">
+        <is>
+          <t>exact_match</t>
+        </is>
+      </c>
+      <c r="O62" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P62" s="4" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="Q62" s="4" t="inlineStr">
+        <is>
+          <t>Brokerage and Commission</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>Jai Kumar Baid</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>AHDPB2654B</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>194H</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="n">
+        <v>17626</v>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H63" s="4" t="n">
+        <v>353</v>
+      </c>
+      <c r="I63" s="4" t="inlineStr">
+        <is>
+          <t>Jai Kumar Baid</t>
+        </is>
+      </c>
+      <c r="J63" s="4" t="n">
+        <v>17626</v>
+      </c>
+      <c r="K63" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="L63" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M63" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N63" s="4" t="inlineStr">
+        <is>
+          <t>exact_match</t>
+        </is>
+      </c>
+      <c r="O63" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P63" s="4" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="Q63" s="4" t="inlineStr">
+        <is>
+          <t>Brokerage and Commission</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>KETAN J SHAH</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>AMUPS0795A</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>194H</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="n">
+        <v>75700</v>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="G64" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H64" s="4" t="n">
+        <v>1514</v>
+      </c>
+      <c r="I64" s="4" t="inlineStr">
+        <is>
+          <t>Ketan Shah</t>
+        </is>
+      </c>
+      <c r="J64" s="4" t="n">
+        <v>75700</v>
+      </c>
+      <c r="K64" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="L64" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M64" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N64" s="4" t="inlineStr">
+        <is>
+          <t>fuzzy_match</t>
+        </is>
+      </c>
+      <c r="O64" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P64" s="4" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="Q64" s="4" t="inlineStr">
+        <is>
+          <t>Brokerage and Commission</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>Kamlesh Kumar Tiwari</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>AEAPT6299J</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>194H</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="n">
+        <v>29484</v>
+      </c>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="G65" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H65" s="4" t="n">
+        <v>590</v>
+      </c>
+      <c r="I65" s="4" t="inlineStr">
+        <is>
+          <t>Kamlesh Kumar Tiwari</t>
+        </is>
+      </c>
+      <c r="J65" s="4" t="n">
+        <v>29484</v>
+      </c>
+      <c r="K65" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="L65" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M65" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N65" s="4" t="inlineStr">
+        <is>
+          <t>exact_match</t>
+        </is>
+      </c>
+      <c r="O65" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P65" s="4" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="Q65" s="4" t="inlineStr">
+        <is>
+          <t>Brokerage and Commission</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>NURPRIT KAUR</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>DPRPK3806R</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>194H</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="n">
+        <v>510428</v>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="G66" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H66" s="4" t="n">
+        <v>10209</v>
+      </c>
+      <c r="I66" s="4" t="inlineStr">
+        <is>
+          <t>Nurprit Kaur</t>
+        </is>
+      </c>
+      <c r="J66" s="4" t="n">
+        <v>510428</v>
+      </c>
+      <c r="K66" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="L66" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M66" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N66" s="4" t="inlineStr">
+        <is>
+          <t>exact_match</t>
+        </is>
+      </c>
+      <c r="O66" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P66" s="4" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="Q66" s="4" t="inlineStr">
+        <is>
+          <t>Brokerage and Commission</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>Rajesh Pandey</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>AIVPP2797G</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>194H</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="n">
+        <v>19608</v>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H67" s="4" t="n">
+        <v>392</v>
+      </c>
+      <c r="I67" s="4" t="inlineStr">
+        <is>
+          <t>Rajesh Pandey</t>
+        </is>
+      </c>
+      <c r="J67" s="4" t="n">
+        <v>19608</v>
+      </c>
+      <c r="K67" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="L67" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M67" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N67" s="4" t="inlineStr">
+        <is>
+          <t>exact_match</t>
+        </is>
+      </c>
+      <c r="O67" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P67" s="4" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="Q67" s="4" t="inlineStr">
+        <is>
+          <t>Brokerage and Commission</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>Tarun Kanti Bhattacharjee</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>ADXPB3392C</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>194H</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="n">
+        <v>16502</v>
+      </c>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="G68" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H68" s="4" t="n">
+        <v>330</v>
+      </c>
+      <c r="I68" s="4" t="inlineStr">
+        <is>
+          <t>Tarun Kanti Bhattacharjee</t>
+        </is>
+      </c>
+      <c r="J68" s="4" t="n">
+        <v>16502</v>
+      </c>
+      <c r="K68" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="L68" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M68" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N68" s="4" t="inlineStr">
+        <is>
+          <t>exact_match</t>
+        </is>
+      </c>
+      <c r="O68" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P68" s="4" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="Q68" s="4" t="inlineStr">
+        <is>
+          <t>Brokerage and Commission</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>VIPUL MANTRI</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>ASYPM7947A</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>194H</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="n">
+        <v>44585</v>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="G69" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H69" s="4" t="n">
+        <v>892</v>
+      </c>
+      <c r="I69" s="4" t="inlineStr">
+        <is>
+          <t>Vipul Mantri</t>
+        </is>
+      </c>
+      <c r="J69" s="4" t="n">
+        <v>44585</v>
+      </c>
+      <c r="K69" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="L69" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M69" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N69" s="4" t="inlineStr">
+        <is>
+          <t>exact_match</t>
+        </is>
+      </c>
+      <c r="O69" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P69" s="4" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="Q69" s="4" t="inlineStr">
+        <is>
+          <t>Brokerage and Commission</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>Vikas Arora</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>ALJPA4325J</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>194H</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="n">
+        <v>64048</v>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="G70" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H70" s="4" t="n">
+        <v>1281</v>
+      </c>
+      <c r="I70" s="4" t="inlineStr">
+        <is>
+          <t>Vikas Arora</t>
+        </is>
+      </c>
+      <c r="J70" s="4" t="n">
+        <v>64048</v>
+      </c>
+      <c r="K70" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="L70" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M70" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N70" s="4" t="inlineStr">
+        <is>
+          <t>exact_match</t>
+        </is>
+      </c>
+      <c r="O70" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P70" s="4" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="Q70" s="4" t="inlineStr">
+        <is>
+          <t>Brokerage and Commission</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>GST PROFESSIONALS LLP</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>AAPFG3370E</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>194J(b)</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="n">
+        <v>31500</v>
+      </c>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="G71" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H71" s="4" t="n">
+        <v>3150</v>
+      </c>
+      <c r="I71" s="4" t="inlineStr">
+        <is>
+          <t>GST Professionals LLP</t>
+        </is>
+      </c>
+      <c r="J71" s="4" t="n">
+        <v>31500</v>
+      </c>
+      <c r="K71" s="4" t="inlineStr">
+        <is>
+          <t>2024-11-30</t>
+        </is>
+      </c>
+      <c r="L71" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M71" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N71" s="4" t="inlineStr">
+        <is>
+          <t>aggregated_cumulative</t>
+        </is>
+      </c>
+      <c r="O71" s="4" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="P71" s="4" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="Q71" s="4" t="inlineStr">
+        <is>
+          <t>Professonal Charges</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>SAHIB S CHOUDHARY &amp; COMPANY</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>AEJPC0634D</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>194J(b)</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="n">
+        <v>9000</v>
+      </c>
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t>2025-01-31</t>
+        </is>
+      </c>
+      <c r="G72" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H72" s="4" t="n">
+        <v>900</v>
+      </c>
+      <c r="I72" s="4" t="inlineStr">
+        <is>
+          <t>Sahib S Choudhary &amp; Co.</t>
+        </is>
+      </c>
+      <c r="J72" s="4" t="n">
+        <v>9000</v>
+      </c>
+      <c r="K72" s="4" t="inlineStr">
+        <is>
+          <t>2025-01-07</t>
+        </is>
+      </c>
+      <c r="L72" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M72" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N72" s="4" t="inlineStr">
+        <is>
+          <t>fuzzy_match</t>
+        </is>
+      </c>
+      <c r="O72" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P72" s="4" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="Q72" s="4" t="inlineStr">
+        <is>
+          <t>GST Annual Return Charges</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>SNCL BUILDERS LLP</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>ADXFS1033K</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>194J(b)</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="n">
+        <v>120000</v>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="G73" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H73" s="4" t="n">
+        <v>12000</v>
+      </c>
+      <c r="I73" s="4" t="inlineStr">
+        <is>
+          <t>SNCL Builders LLP</t>
+        </is>
+      </c>
+      <c r="J73" s="4" t="n">
+        <v>120000</v>
+      </c>
+      <c r="K73" s="4" t="inlineStr">
+        <is>
+          <t>2024-12-05</t>
+        </is>
+      </c>
+      <c r="L73" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M73" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N73" s="4" t="inlineStr">
+        <is>
+          <t>fuzzy_match</t>
+        </is>
+      </c>
+      <c r="O73" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P73" s="4" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="Q73" s="4" t="inlineStr">
+        <is>
+          <t>Consultancy Charges</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>RAYMOND LIFESTYLE LTD.</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>AAJCR2207E</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>194Q</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="n">
+        <v>14544442</v>
+      </c>
+      <c r="F74" s="4" t="inlineStr">
+        <is>
+          <t>2024-09-30</t>
+        </is>
+      </c>
+      <c r="G74" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H74" s="4" t="n">
+        <v>14544</v>
+      </c>
+      <c r="I74" s="4" t="inlineStr">
+        <is>
+          <t>Raymond Lifestyle Limited (Shirting Div.)</t>
+        </is>
+      </c>
+      <c r="J74" s="4" t="n">
+        <v>14544448</v>
+      </c>
+      <c r="K74" s="4" t="inlineStr">
+        <is>
+          <t>2024-09-28</t>
+        </is>
+      </c>
+      <c r="L74" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M74" s="4" t="n">
+        <v>-6</v>
+      </c>
+      <c r="N74" s="4" t="inlineStr">
+        <is>
+          <t>fuzzy_match</t>
+        </is>
+      </c>
+      <c r="O74" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P74" s="4" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="Q74" s="4" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>RAYMOND LIFESTYLE LTD.</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>AAJCR2207E</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>194Q</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="n">
+        <v>2462522</v>
+      </c>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>2024-10-31</t>
+        </is>
+      </c>
+      <c r="G75" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H75" s="4" t="n">
+        <v>2463</v>
+      </c>
+      <c r="I75" s="4" t="inlineStr">
+        <is>
+          <t>Raymond Lifestyle Limited (Shirting Div.)</t>
+        </is>
+      </c>
+      <c r="J75" s="4" t="n">
+        <v>2462521</v>
+      </c>
+      <c r="K75" s="4" t="inlineStr">
+        <is>
+          <t>2024-10-28</t>
+        </is>
+      </c>
+      <c r="L75" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M75" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N75" s="4" t="inlineStr">
+        <is>
+          <t>fuzzy_match</t>
+        </is>
+      </c>
+      <c r="O75" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P75" s="4" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="Q75" s="4" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>RAYMOND LIFESTYLE LTD.</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>AAJCR2207E</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>194Q</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="n">
+        <v>13796210</v>
+      </c>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="G76" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H76" s="4" t="n">
+        <v>13796</v>
+      </c>
+      <c r="I76" s="4" t="inlineStr">
+        <is>
+          <t>Raymond Lifestyle Limited (Shirting Div.)</t>
+        </is>
+      </c>
+      <c r="J76" s="4" t="n">
+        <v>13796210</v>
+      </c>
+      <c r="K76" s="4" t="inlineStr">
+        <is>
+          <t>2024-12-28</t>
+        </is>
+      </c>
+      <c r="L76" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M76" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N76" s="4" t="inlineStr">
+        <is>
+          <t>exact_match</t>
+        </is>
+      </c>
+      <c r="O76" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P76" s="4" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="Q76" s="4" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>RAYMOND LIFESTYLE LTD.</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>AAJCR2207E</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>194Q</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="n">
+        <v>5947729</v>
+      </c>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>2025-01-31</t>
+        </is>
+      </c>
+      <c r="G77" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H77" s="4" t="n">
+        <v>5948</v>
+      </c>
+      <c r="I77" s="4" t="inlineStr">
+        <is>
+          <t>Raymond Lifestyle Limited (Shirting Div.)</t>
+        </is>
+      </c>
+      <c r="J77" s="4" t="n">
+        <v>5947728</v>
+      </c>
+      <c r="K77" s="4" t="inlineStr">
+        <is>
+          <t>2025-01-28</t>
+        </is>
+      </c>
+      <c r="L77" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M77" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N77" s="4" t="inlineStr">
+        <is>
+          <t>fuzzy_match</t>
+        </is>
+      </c>
+      <c r="O77" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P77" s="4" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="Q77" s="4" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>RAYMOND LIFESTYLE LTD.</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>AAJCR2207E</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>194Q</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="n">
+        <v>7934577</v>
+      </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="G78" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H78" s="4" t="n">
+        <v>7935</v>
+      </c>
+      <c r="I78" s="4" t="inlineStr">
+        <is>
+          <t>Raymond Lifestyle Limited (Shirting Div.)</t>
+        </is>
+      </c>
+      <c r="J78" s="4" t="n">
+        <v>7934577</v>
+      </c>
+      <c r="K78" s="4" t="inlineStr">
+        <is>
+          <t>2025-03-28</t>
+        </is>
+      </c>
+      <c r="L78" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M78" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N78" s="4" t="inlineStr">
+        <is>
+          <t>exact_match</t>
+        </is>
+      </c>
+      <c r="O78" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P78" s="4" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="Q78" s="4" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>Raymond Limited</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>AAACR4896A</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>194Q</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="n">
+        <v>1480982</v>
+      </c>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>2024-06-30</t>
+        </is>
+      </c>
+      <c r="G79" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H79" s="4" t="n">
+        <v>1481</v>
+      </c>
+      <c r="I79" s="4" t="inlineStr">
+        <is>
+          <t>Raymond Limited (Shirting Division)</t>
+        </is>
+      </c>
+      <c r="J79" s="4" t="n">
+        <v>1480982</v>
+      </c>
+      <c r="K79" s="4" t="inlineStr">
+        <is>
+          <t>2024-06-28</t>
+        </is>
+      </c>
+      <c r="L79" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M79" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N79" s="4" t="inlineStr">
+        <is>
+          <t>exact_match</t>
+        </is>
+      </c>
+      <c r="O79" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P79" s="4" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="Q79" s="4" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>Sai Boutique</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>AEPFS3230M</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>194Q</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="n">
+        <v>381820</v>
+      </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>2025-01-31</t>
+        </is>
+      </c>
+      <c r="G80" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H80" s="4" t="n">
+        <v>382</v>
+      </c>
+      <c r="I80" s="4" t="inlineStr">
+        <is>
+          <t>Sai Boutique</t>
+        </is>
+      </c>
+      <c r="J80" s="4" t="n">
+        <v>381820</v>
+      </c>
+      <c r="K80" s="4" t="inlineStr">
+        <is>
+          <t>2025-01-28</t>
+        </is>
+      </c>
+      <c r="L80" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N80" s="4" t="inlineStr">
+        <is>
+          <t>exact_match</t>
+        </is>
+      </c>
+      <c r="O80" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P80" s="4" t="inlineStr">
+        <is>
+          <t>Reconciled</t>
+        </is>
+      </c>
+      <c r="Q80" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q57"/>
+  <autoFilter ref="A1:Q80"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5077,7 +6872,7 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 63,000 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 63,000 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -5108,7 +6903,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 39,830 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 39,830 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -5139,7 +6934,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 39,000 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 39,000 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -5170,7 +6965,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 38,743 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 38,743 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -5201,7 +6996,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 31,645 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 31,645 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -5232,7 +7027,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 31,160 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 31,160 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -5263,7 +7058,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 25,600 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 25,600 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -5294,7 +7089,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 25,489 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 25,489 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -5325,7 +7120,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 22,944 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 22,944 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -5356,7 +7151,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 22,308 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 22,308 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -5387,7 +7182,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 20,988 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 20,988 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -5418,7 +7213,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 20,800 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 20,800 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -5449,7 +7244,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 20,762 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 20,762 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -5480,7 +7275,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 20,048 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 20,048 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -5511,7 +7306,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 19,316 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 19,316 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -5542,7 +7337,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 18,409 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 18,409 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -5573,7 +7368,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 17,633 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 17,633 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -5604,7 +7399,7 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 15,488 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 15,488 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -5635,7 +7430,7 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 14,642 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 14,642 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -5666,7 +7461,7 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 12,802 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 12,802 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -5697,7 +7492,7 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 10,670 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 10,670 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -5728,7 +7523,7 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 9,976 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 9,976 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -5759,7 +7554,7 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 9,307 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 9,307 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -5790,7 +7585,7 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 7,143 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 7,143 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -5821,7 +7616,7 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 7,023 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 7,023 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -5852,7 +7647,7 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 6,791 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 6,791 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -5883,7 +7678,7 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 6,102 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 6,102 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -5914,7 +7709,7 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 6,000 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 6,000 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -5945,7 +7740,7 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 6,000 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 6,000 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -5976,7 +7771,7 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 5,825 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 5,825 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -6007,7 +7802,7 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 5,700 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 5,700 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -6038,7 +7833,7 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 5,339 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 5,339 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -6069,7 +7864,7 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 5,045 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 5,045 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -6100,7 +7895,7 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 4,950 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 4,950 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -6131,7 +7926,7 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 4,735 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 4,735 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -6162,7 +7957,7 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 4,305 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 4,305 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -6193,7 +7988,7 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 4,121 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 4,121 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -6224,7 +8019,7 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 3,759 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 3,759 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
@@ -6255,7 +8050,7 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 3,573 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 3,573 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -6286,7 +8081,7 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 3,380 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 3,380 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
@@ -6317,7 +8112,7 @@
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 3,200 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 3,200 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -6348,7 +8143,7 @@
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 2,700 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 2,700 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
@@ -6379,7 +8174,7 @@
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 2,699 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 2,699 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
@@ -6410,7 +8205,7 @@
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 2,142 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 2,142 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
@@ -6441,7 +8236,7 @@
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 1,880 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 1,880 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
@@ -6472,7 +8267,7 @@
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 1,500 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 1,500 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
@@ -6503,7 +8298,7 @@
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 1,428 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 1,428 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -6534,7 +8329,7 @@
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 1,346 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 1,346 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
@@ -6565,7 +8360,7 @@
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 964 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 964 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
@@ -6596,7 +8391,7 @@
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 930 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 930 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
@@ -6627,7 +8422,7 @@
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 762 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 762 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
@@ -6658,7 +8453,7 @@
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 723 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 723 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
@@ -6689,7 +8484,7 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 623 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 623 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
@@ -6720,7 +8515,7 @@
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 600 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 600 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
@@ -6751,7 +8546,7 @@
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 480 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 480 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
@@ -6782,7 +8577,7 @@
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 450 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 450 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
@@ -6813,7 +8608,7 @@
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 326 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 326 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
@@ -6844,7 +8639,7 @@
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 318 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 318 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
@@ -6875,7 +8670,7 @@
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>Below threshold - aggregate Rs 225 &lt; Rs 1,00,000 annual limit</t>
+          <t>Below threshold - aggregate Rs 225 &lt; ₹1,00,000 annual limit</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Always show timing sheets — positive message when no delays
- Late TDS Deduction + Late TDS Deposit sheets always present in Excel
- When no delays: "✓ All TDS deductions/deposits were made on time. Great compliance!"
- Green bold font for positive message

https://claude.ai/code/session_01U1MuRvDgn4XPQ38Fe5qjWF
</commit_message>
<xml_diff>
--- a/tds-recon/data/results/tds_recon_report.xlsx
+++ b/tds-recon/data/results/tds_recon_report.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TDS Report - Matched" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zero TDS - Exempt" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Late TDS Deduction" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Late TDS Deposit" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Issues for Review'!$A$1:$J$117</definedName>
@@ -25,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,6 +38,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0016A34A"/>
+      <sz val="13"/>
     </font>
   </fonts>
   <fills count="5">
@@ -91,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -105,6 +111,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -19747,4 +19754,28 @@
   <autoFilter ref="A1:N105"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>✓ All TDS deposits were made on time. Great compliance!</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix misleading threshold finding — clarify Form 26 amount vs total books
- threshold_validation now says "Form 26 aggregate" not just "aggregate"
- Adds note: "verify total books expense is also below threshold"
- Only shows below-threshold finding when F26 amount < 50% of threshold
  (avoids contradicting partial_tds finding for same vendor)
- Sahib: threshold INFO now coexists correctly with partial_tds ERROR

https://claude.ai/code/session_01U1MuRvDgn4XPQ38Fe5qjWF
</commit_message>
<xml_diff>
--- a/tds-recon/data/results/tds_recon_report.xlsx
+++ b/tds-recon/data/results/tds_recon_report.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Late TDS Deposit" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Issues for Review'!$A$1:$J$117</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Issues for Review'!$A$1:$J$121</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'TDS Report - Matched'!$A$1:$Q$80</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Zero TDS - Exempt'!$A$1:$G$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Late TDS Deduction'!$A$1:$N$105</definedName>
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J117"/>
+  <dimension ref="A1:J121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -555,26 +555,28 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>partial_tds</t>
+          <t>pan_validation</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Sahib S Choudhary &amp; Co.</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr"/>
+          <t>Adi Debnath</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>AAAAA0001A</t>
+        </is>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>194J(b)</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>30000</v>
-      </c>
+          <t>194A</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Vendor Sahib S Choudhary &amp; Co. has Form 26 entry under 194J(b) but additional ₹30,000 in books (Audit Fees) is not covered. TDS may be short-deducted.</t>
+          <t>Invalid/missing PAN for Adi Debnath — Section 206AA requires TDS at 20.0% (applied 10%). Potential short deduction: ₹8,246.</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -599,7 +601,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>tds_timing</t>
+          <t>pan_validation</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -620,7 +622,7 @@
       <c r="G3" s="2" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on Adi Debnath (194A): Expense on 19-Mar-2025, TDS deducted on 31-Mar-2025 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹88 (8,821 × 1% × 1 months).</t>
+          <t>Invalid/missing PAN for Adi Debnath — Section 206AA requires TDS at 20.0% (applied 10%). Potential short deduction: ₹8,575.</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -645,17 +647,17 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>tds_timing</t>
+          <t>pan_validation</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Asha Negi</t>
+          <t>Adi Debnath</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>AAAAA0002A</t>
+          <t>AAAAA0001A</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -666,7 +668,7 @@
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on Asha Negi (194A): Expense on 19-Mar-2025, TDS deducted on 31-Mar-2025 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹133 (13,315 × 1% × 1 months).</t>
+          <t>Invalid/missing PAN for Adi Debnath — Section 206AA requires TDS at 20.0% (applied 10%). Potential short deduction: ₹8,813.</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -691,17 +693,17 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>tds_timing</t>
+          <t>pan_validation</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Manisha Kumari</t>
+          <t>Adi Debnath</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>AAAAA0003A</t>
+          <t>AAAAA0001A</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -712,7 +714,7 @@
       <c r="G5" s="2" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on Manisha Kumari (194A): Expense on 19-Mar-2025, TDS deducted on 31-Mar-2025 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹261 (26,131 × 1% × 1 months).</t>
+          <t>Invalid/missing PAN for Adi Debnath — Section 206AA requires TDS at 20.0% (applied 10%). Potential short deduction: ₹8,821.</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -737,28 +739,26 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>tds_timing</t>
+          <t>partial_tds</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Suresh Sethia</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>AAAAA0004A</t>
-        </is>
-      </c>
+          <t>Sahib S Choudhary &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>194A</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr"/>
+          <t>194J(b)</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>30000</v>
+      </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on Suresh Sethia (194A): Expense on 19-Mar-2025, TDS deducted on 31-Mar-2025 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹509 (50,930 × 1% × 1 months).</t>
+          <t>Vendor Sahib S Choudhary &amp; Co. has Form 26 entry under 194J(b) but additional ₹30,000 in books (Audit Fees) is not covered. TDS may be short-deducted.</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -788,12 +788,12 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Rupa Khaitan</t>
+          <t>Adi Debnath</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>AAAAA0007A</t>
+          <t>AAAAA0001A</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -804,7 +804,7 @@
       <c r="G7" s="2" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on Rupa Khaitan (194A): Expense on 19-Mar-2025, TDS deducted on 31-Mar-2025 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹21 (2,064 × 1% × 1 months).</t>
+          <t>Late TDS deduction on Adi Debnath (194A): Expense on 19-Mar-2025, TDS deducted on 31-Mar-2025 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹88 (8,821 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -834,12 +834,12 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Akash Nagar</t>
+          <t>Asha Negi</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>AAAAA0005A</t>
+          <t>AAAAA0002A</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -850,7 +850,7 @@
       <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on Akash Nagar (194A): Expense on 19-Mar-2025, TDS deducted on 31-Mar-2025 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹491 (49,099 × 1% × 1 months).</t>
+          <t>Late TDS deduction on Asha Negi (194A): Expense on 19-Mar-2025, TDS deducted on 31-Mar-2025 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹133 (13,315 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -880,12 +880,12 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Rahul Shah</t>
+          <t>Manisha Kumari</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>AAAAA0006A</t>
+          <t>AAAAA0003A</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -896,7 +896,7 @@
       <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on Rahul Shah (194A): Expense on 19-Mar-2025, TDS deducted on 31-Mar-2025 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹206 (20,593 × 1% × 1 months).</t>
+          <t>Late TDS deduction on Manisha Kumari (194A): Expense on 19-Mar-2025, TDS deducted on 31-Mar-2025 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹261 (26,131 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -926,12 +926,12 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Karan Kothari</t>
+          <t>Suresh Sethia</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>AAAAA0008A</t>
+          <t>AAAAA0004A</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -942,7 +942,7 @@
       <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on Karan Kothari (194A): Expense on 19-Mar-2025, TDS deducted on 31-Mar-2025 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹153 (15,312 × 1% × 1 months).</t>
+          <t>Late TDS deduction on Suresh Sethia (194A): Expense on 19-Mar-2025, TDS deducted on 31-Mar-2025 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹509 (50,930 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -972,12 +972,12 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Ramesh Lohia</t>
+          <t>Rupa Khaitan</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>AAAAA0009A</t>
+          <t>AAAAA0007A</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -988,7 +988,7 @@
       <c r="G11" s="2" t="inlineStr"/>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on Ramesh Lohia (194A): Expense on 19-Mar-2025, TDS deducted on 31-Mar-2025 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹80 (7,989 × 1% × 1 months).</t>
+          <t>Late TDS deduction on Rupa Khaitan (194A): Expense on 19-Mar-2025, TDS deducted on 31-Mar-2025 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹21 (2,064 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1018,23 +1018,23 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>AMRITA ICONS</t>
+          <t>Akash Nagar</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>AYBPS6260R</t>
+          <t>AAAAA0005A</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>194C</t>
+          <t>194A</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on AMRITA ICONS (194C): Expense on 28-May-2024, TDS deducted on 30-Sep-2024 (125 days late, 5 month(s)). Interest u/s 201(1A): ₹1 (16 × 1% × 5 months).</t>
+          <t>Late TDS deduction on Akash Nagar (194A): Expense on 19-Mar-2025, TDS deducted on 31-Mar-2025 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹491 (49,099 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1064,23 +1064,23 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>AMRITA ICONS</t>
+          <t>Rahul Shah</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>AYBPS6260R</t>
+          <t>AAAAA0006A</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>194C</t>
+          <t>194A</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on AMRITA ICONS (194C): Expense on 05-Sep-2024, TDS deducted on 30-Sep-2024 (25 days late, 1 month(s)). Interest u/s 201(1A): ₹18 (1,798 × 1% × 1 months).</t>
+          <t>Late TDS deduction on Rahul Shah (194A): Expense on 19-Mar-2025, TDS deducted on 31-Mar-2025 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹206 (20,593 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1110,23 +1110,23 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>AMRITA ICONS</t>
+          <t>Karan Kothari</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>AYBPS6260R</t>
+          <t>AAAAA0008A</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>194C</t>
+          <t>194A</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on AMRITA ICONS (194C): Expense on 06-Mar-2025, TDS deducted on 31-Mar-2025 (25 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (17 × 1% × 1 months).</t>
+          <t>Late TDS deduction on Karan Kothari (194A): Expense on 19-Mar-2025, TDS deducted on 31-Mar-2025 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹153 (15,312 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1156,23 +1156,23 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>AMRITA ICONS</t>
+          <t>Ramesh Lohia</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>AYBPS6260R</t>
+          <t>AAAAA0009A</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>194C</t>
+          <t>194A</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr"/>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on AMRITA ICONS (194C): Expense on 28-Mar-2025, TDS deducted on 31-Mar-2025 (3 days late, 1 month(s)). Interest u/s 201(1A): ₹2 (236 × 1% × 1 months).</t>
+          <t>Late TDS deduction on Ramesh Lohia (194A): Expense on 19-Mar-2025, TDS deducted on 31-Mar-2025 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹80 (7,989 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1202,12 +1202,12 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>ANDERSON TECHNOLOGY PVT LTD</t>
+          <t>AMRITA ICONS</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>AAFCA4805K</t>
+          <t>AYBPS6260R</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1218,7 +1218,7 @@
       <c r="G16" s="2" t="inlineStr"/>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on ANDERSON TECHNOLOGY PVT LTD (194C): Expense on 30-Sep-2024, TDS deducted on 31-Jan-2025 (123 days late, 5 month(s)). Interest u/s 201(1A): ₹70 (1,400 × 1% × 5 months).</t>
+          <t>Late TDS deduction on AMRITA ICONS (194C): Expense on 28-May-2024, TDS deducted on 30-Sep-2024 (125 days late, 5 month(s)). Interest u/s 201(1A): ₹1 (16 × 1% × 5 months).</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1248,12 +1248,12 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>ANDERSON TECHNOLOGY PVT LTD</t>
+          <t>AMRITA ICONS</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>AAFCA4805K</t>
+          <t>AYBPS6260R</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1264,7 +1264,7 @@
       <c r="G17" s="2" t="inlineStr"/>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on ANDERSON TECHNOLOGY PVT LTD (194C): Expense on 31-Oct-2024, TDS deducted on 31-Jan-2025 (92 days late, 4 month(s)). Interest u/s 201(1A): ₹3 (67 × 1% × 4 months).</t>
+          <t>Late TDS deduction on AMRITA ICONS (194C): Expense on 05-Sep-2024, TDS deducted on 30-Sep-2024 (25 days late, 1 month(s)). Interest u/s 201(1A): ₹18 (1,798 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1294,12 +1294,12 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>ANDERSON TECHNOLOGY PVT LTD</t>
+          <t>AMRITA ICONS</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>AAFCA4805K</t>
+          <t>AYBPS6260R</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1310,7 +1310,7 @@
       <c r="G18" s="2" t="inlineStr"/>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on ANDERSON TECHNOLOGY PVT LTD (194C): Expense on 31-Oct-2024, TDS deducted on 31-Jan-2025 (92 days late, 4 month(s)). Interest u/s 201(1A): ₹3 (67 × 1% × 4 months).</t>
+          <t>Late TDS deduction on AMRITA ICONS (194C): Expense on 06-Mar-2025, TDS deducted on 31-Mar-2025 (25 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (17 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1340,12 +1340,12 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>ANDERSON TECHNOLOGY PVT LTD</t>
+          <t>AMRITA ICONS</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>AAFCA4805K</t>
+          <t>AYBPS6260R</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1356,7 +1356,7 @@
       <c r="G19" s="2" t="inlineStr"/>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on ANDERSON TECHNOLOGY PVT LTD (194C): Expense on 30-Nov-2024, TDS deducted on 31-Jan-2025 (62 days late, 3 month(s)). Interest u/s 201(1A): ₹9 (300 × 1% × 3 months).</t>
+          <t>Late TDS deduction on AMRITA ICONS (194C): Expense on 28-Mar-2025, TDS deducted on 31-Mar-2025 (3 days late, 1 month(s)). Interest u/s 201(1A): ₹2 (236 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -1402,7 +1402,7 @@
       <c r="G20" s="2" t="inlineStr"/>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on ANDERSON TECHNOLOGY PVT LTD (194C): Expense on 30-Nov-2024, TDS deducted on 31-Jan-2025 (62 days late, 3 month(s)). Interest u/s 201(1A): ₹2 (67 × 1% × 3 months).</t>
+          <t>Late TDS deduction on ANDERSON TECHNOLOGY PVT LTD (194C): Expense on 30-Sep-2024, TDS deducted on 31-Jan-2025 (123 days late, 5 month(s)). Interest u/s 201(1A): ₹70 (1,400 × 1% × 5 months).</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -1448,7 +1448,7 @@
       <c r="G21" s="2" t="inlineStr"/>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on ANDERSON TECHNOLOGY PVT LTD (194C): Expense on 31-Dec-2024, TDS deducted on 31-Jan-2025 (31 days late, 2 month(s)). Interest u/s 201(1A): ₹1 (67 × 1% × 2 months).</t>
+          <t>Late TDS deduction on ANDERSON TECHNOLOGY PVT LTD (194C): Expense on 31-Oct-2024, TDS deducted on 31-Jan-2025 (92 days late, 4 month(s)). Interest u/s 201(1A): ₹3 (67 × 1% × 4 months).</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -1494,7 +1494,7 @@
       <c r="G22" s="2" t="inlineStr"/>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on ANDERSON TECHNOLOGY PVT LTD (194C): Expense on 16-Jan-2025, TDS deducted on 31-Jan-2025 (15 days late, 1 month(s)). Interest u/s 201(1A): ₹7 (720 × 1% × 1 months).</t>
+          <t>Late TDS deduction on ANDERSON TECHNOLOGY PVT LTD (194C): Expense on 31-Oct-2024, TDS deducted on 31-Jan-2025 (92 days late, 4 month(s)). Interest u/s 201(1A): ₹3 (67 × 1% × 4 months).</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1540,7 +1540,7 @@
       <c r="G23" s="2" t="inlineStr"/>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on ANDERSON TECHNOLOGY PVT LTD (194C): Expense on 31-Jan-2025, TDS deducted on 28-Feb-2025 (28 days late, 1 month(s)). Interest u/s 201(1A): ₹1 (66 × 1% × 1 months).</t>
+          <t>Late TDS deduction on ANDERSON TECHNOLOGY PVT LTD (194C): Expense on 30-Nov-2024, TDS deducted on 31-Jan-2025 (62 days late, 3 month(s)). Interest u/s 201(1A): ₹9 (300 × 1% × 3 months).</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -1586,7 +1586,7 @@
       <c r="G24" s="2" t="inlineStr"/>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on ANDERSON TECHNOLOGY PVT LTD (194C): Expense on 28-Feb-2025, TDS deducted on 01-Mar-2025 (1 days late, 1 month(s)). Interest u/s 201(1A): ₹8 (800 × 1% × 1 months).</t>
+          <t>Late TDS deduction on ANDERSON TECHNOLOGY PVT LTD (194C): Expense on 30-Nov-2024, TDS deducted on 31-Jan-2025 (62 days late, 3 month(s)). Interest u/s 201(1A): ₹2 (67 × 1% × 3 months).</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -1616,12 +1616,12 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>ANDREAL INNOVATION PVT LTD</t>
+          <t>ANDERSON TECHNOLOGY PVT LTD</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>ABACA2255R</t>
+          <t>AAFCA4805K</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1632,7 +1632,7 @@
       <c r="G25" s="2" t="inlineStr"/>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on ANDREAL INNOVATION PVT LTD (194C): Expense on 13-Jul-2024, TDS deducted on 01-Mar-2025 (231 days late, 8 month(s)). Interest u/s 201(1A): ₹40 (500 × 1% × 8 months).</t>
+          <t>Late TDS deduction on ANDERSON TECHNOLOGY PVT LTD (194C): Expense on 31-Dec-2024, TDS deducted on 31-Jan-2025 (31 days late, 2 month(s)). Interest u/s 201(1A): ₹1 (67 × 1% × 2 months).</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -1662,12 +1662,12 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>ANDREAL INNOVATION PVT LTD</t>
+          <t>ANDERSON TECHNOLOGY PVT LTD</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>ABACA2255R</t>
+          <t>AAFCA4805K</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1678,7 +1678,7 @@
       <c r="G26" s="2" t="inlineStr"/>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on ANDREAL INNOVATION PVT LTD (194C): Expense on 13-Jul-2024, TDS deducted on 01-Mar-2025 (231 days late, 8 month(s)). Interest u/s 201(1A): ₹48 (600 × 1% × 8 months).</t>
+          <t>Late TDS deduction on ANDERSON TECHNOLOGY PVT LTD (194C): Expense on 16-Jan-2025, TDS deducted on 31-Jan-2025 (15 days late, 1 month(s)). Interest u/s 201(1A): ₹7 (720 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -1708,12 +1708,12 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>ANDREAL INNOVATION PVT LTD</t>
+          <t>ANDERSON TECHNOLOGY PVT LTD</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>ABACA2255R</t>
+          <t>AAFCA4805K</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1724,7 +1724,7 @@
       <c r="G27" s="2" t="inlineStr"/>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on ANDREAL INNOVATION PVT LTD (194C): Expense on 31-Jul-2024, TDS deducted on 01-Mar-2025 (213 days late, 8 month(s)). Interest u/s 201(1A): ₹18 (230 × 1% × 8 months).</t>
+          <t>Late TDS deduction on ANDERSON TECHNOLOGY PVT LTD (194C): Expense on 31-Jan-2025, TDS deducted on 28-Feb-2025 (28 days late, 1 month(s)). Interest u/s 201(1A): ₹1 (66 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -1754,12 +1754,12 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>ANDREAL INNOVATION PVT LTD</t>
+          <t>ANDERSON TECHNOLOGY PVT LTD</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>ABACA2255R</t>
+          <t>AAFCA4805K</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1770,7 +1770,7 @@
       <c r="G28" s="2" t="inlineStr"/>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on ANDREAL INNOVATION PVT LTD (194C): Expense on 04-Feb-2025, TDS deducted on 01-Mar-2025 (25 days late, 1 month(s)). Interest u/s 201(1A): ₹3 (300 × 1% × 1 months).</t>
+          <t>Late TDS deduction on ANDERSON TECHNOLOGY PVT LTD (194C): Expense on 28-Feb-2025, TDS deducted on 01-Mar-2025 (1 days late, 1 month(s)). Interest u/s 201(1A): ₹8 (800 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -1800,12 +1800,12 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>INLAND WORLD LOGISTICS PVT LTD</t>
+          <t>ANDREAL INNOVATION PVT LTD</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>AAACI5607C</t>
+          <t>ABACA2255R</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1816,7 +1816,7 @@
       <c r="G29" s="2" t="inlineStr"/>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 04-Apr-2024, TDS deducted on 30-Apr-2024 (26 days late, 1 month(s)). Interest u/s 201(1A): ₹4 (450 × 1% × 1 months).</t>
+          <t>Late TDS deduction on ANDREAL INNOVATION PVT LTD (194C): Expense on 13-Jul-2024, TDS deducted on 01-Mar-2025 (231 days late, 8 month(s)). Interest u/s 201(1A): ₹40 (500 × 1% × 8 months).</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -1846,12 +1846,12 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>INLAND WORLD LOGISTICS PVT LTD</t>
+          <t>ANDREAL INNOVATION PVT LTD</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>AAACI5607C</t>
+          <t>ABACA2255R</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -1862,7 +1862,7 @@
       <c r="G30" s="2" t="inlineStr"/>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 04-Apr-2024, TDS deducted on 30-Apr-2024 (26 days late, 1 month(s)). Interest u/s 201(1A): ₹2 (224 × 1% × 1 months).</t>
+          <t>Late TDS deduction on ANDREAL INNOVATION PVT LTD (194C): Expense on 13-Jul-2024, TDS deducted on 01-Mar-2025 (231 days late, 8 month(s)). Interest u/s 201(1A): ₹48 (600 × 1% × 8 months).</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -1892,12 +1892,12 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>INLAND WORLD LOGISTICS PVT LTD</t>
+          <t>ANDREAL INNOVATION PVT LTD</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>AAACI5607C</t>
+          <t>ABACA2255R</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -1908,7 +1908,7 @@
       <c r="G31" s="2" t="inlineStr"/>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 16-May-2024, TDS deducted on 31-May-2024 (15 days late, 1 month(s)). Interest u/s 201(1A): ₹1 (133 × 1% × 1 months).</t>
+          <t>Late TDS deduction on ANDREAL INNOVATION PVT LTD (194C): Expense on 31-Jul-2024, TDS deducted on 01-Mar-2025 (213 days late, 8 month(s)). Interest u/s 201(1A): ₹18 (230 × 1% × 8 months).</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -1938,12 +1938,12 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>INLAND WORLD LOGISTICS PVT LTD</t>
+          <t>ANDREAL INNOVATION PVT LTD</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>AAACI5607C</t>
+          <t>ABACA2255R</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -1954,7 +1954,7 @@
       <c r="G32" s="2" t="inlineStr"/>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 30-May-2024, TDS deducted on 31-May-2024 (1 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (33 × 1% × 1 months).</t>
+          <t>Late TDS deduction on ANDREAL INNOVATION PVT LTD (194C): Expense on 04-Feb-2025, TDS deducted on 01-Mar-2025 (25 days late, 1 month(s)). Interest u/s 201(1A): ₹3 (300 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -2000,7 +2000,7 @@
       <c r="G33" s="2" t="inlineStr"/>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 30-May-2024, TDS deducted on 31-May-2024 (1 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (11 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 04-Apr-2024, TDS deducted on 30-Apr-2024 (26 days late, 1 month(s)). Interest u/s 201(1A): ₹4 (450 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -2046,7 +2046,7 @@
       <c r="G34" s="2" t="inlineStr"/>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 18-Jun-2024, TDS deducted on 30-Jun-2024 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (11 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 04-Apr-2024, TDS deducted on 30-Apr-2024 (26 days late, 1 month(s)). Interest u/s 201(1A): ₹2 (224 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -2092,7 +2092,7 @@
       <c r="G35" s="2" t="inlineStr"/>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 18-Jun-2024, TDS deducted on 30-Jun-2024 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹9 (858 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 16-May-2024, TDS deducted on 31-May-2024 (15 days late, 1 month(s)). Interest u/s 201(1A): ₹1 (133 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -2138,7 +2138,7 @@
       <c r="G36" s="2" t="inlineStr"/>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 22-Jun-2024, TDS deducted on 30-Jun-2024 (8 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (25 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 30-May-2024, TDS deducted on 31-May-2024 (1 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (33 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -2184,7 +2184,7 @@
       <c r="G37" s="2" t="inlineStr"/>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 03-Jul-2024, TDS deducted on 31-Jul-2024 (28 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (11 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 30-May-2024, TDS deducted on 31-May-2024 (1 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (11 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
@@ -2230,7 +2230,7 @@
       <c r="G38" s="2" t="inlineStr"/>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 03-Jul-2024, TDS deducted on 31-Jul-2024 (28 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (12 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 18-Jun-2024, TDS deducted on 30-Jun-2024 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (11 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -2276,7 +2276,7 @@
       <c r="G39" s="2" t="inlineStr"/>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 03-Jul-2024, TDS deducted on 31-Jul-2024 (28 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (12 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 18-Jun-2024, TDS deducted on 30-Jun-2024 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹9 (858 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
@@ -2322,7 +2322,7 @@
       <c r="G40" s="2" t="inlineStr"/>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 03-Jul-2024, TDS deducted on 31-Jul-2024 (28 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (6 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 22-Jun-2024, TDS deducted on 30-Jun-2024 (8 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (25 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -2368,7 +2368,7 @@
       <c r="G41" s="2" t="inlineStr"/>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 03-Jul-2024, TDS deducted on 31-Jul-2024 (28 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (6 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 03-Jul-2024, TDS deducted on 31-Jul-2024 (28 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (11 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -2414,7 +2414,7 @@
       <c r="G42" s="2" t="inlineStr"/>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 12-Jul-2024, TDS deducted on 31-Jul-2024 (19 days late, 1 month(s)). Interest u/s 201(1A): ₹1 (76 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 03-Jul-2024, TDS deducted on 31-Jul-2024 (28 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (12 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
@@ -2460,7 +2460,7 @@
       <c r="G43" s="2" t="inlineStr"/>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 12-Jul-2024, TDS deducted on 31-Jul-2024 (19 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (39 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 03-Jul-2024, TDS deducted on 31-Jul-2024 (28 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (12 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
@@ -2506,7 +2506,7 @@
       <c r="G44" s="2" t="inlineStr"/>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 12-Jul-2024, TDS deducted on 31-Jul-2024 (19 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (36 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 03-Jul-2024, TDS deducted on 31-Jul-2024 (28 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (6 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
@@ -2552,7 +2552,7 @@
       <c r="G45" s="2" t="inlineStr"/>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 25-Jul-2024, TDS deducted on 31-Jul-2024 (6 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (14 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 03-Jul-2024, TDS deducted on 31-Jul-2024 (28 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (6 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
@@ -2598,7 +2598,7 @@
       <c r="G46" s="2" t="inlineStr"/>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 02-Aug-2024, TDS deducted on 31-Aug-2024 (29 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (13 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 12-Jul-2024, TDS deducted on 31-Jul-2024 (19 days late, 1 month(s)). Interest u/s 201(1A): ₹1 (76 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
@@ -2644,7 +2644,7 @@
       <c r="G47" s="2" t="inlineStr"/>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 05-Aug-2024, TDS deducted on 31-Aug-2024 (26 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (8 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 12-Jul-2024, TDS deducted on 31-Jul-2024 (19 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (39 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
@@ -2690,7 +2690,7 @@
       <c r="G48" s="2" t="inlineStr"/>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 05-Aug-2024, TDS deducted on 31-Aug-2024 (26 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (6 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 12-Jul-2024, TDS deducted on 31-Jul-2024 (19 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (36 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
@@ -2736,7 +2736,7 @@
       <c r="G49" s="2" t="inlineStr"/>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 16-Aug-2024, TDS deducted on 31-Aug-2024 (15 days late, 1 month(s)). Interest u/s 201(1A): ₹2 (205 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 25-Jul-2024, TDS deducted on 31-Jul-2024 (6 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (14 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
@@ -2782,7 +2782,7 @@
       <c r="G50" s="2" t="inlineStr"/>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 16-Aug-2024, TDS deducted on 31-Aug-2024 (15 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (28 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 02-Aug-2024, TDS deducted on 31-Aug-2024 (29 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (13 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
@@ -2828,7 +2828,7 @@
       <c r="G51" s="2" t="inlineStr"/>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 16-Aug-2024, TDS deducted on 31-Aug-2024 (15 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (11 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 05-Aug-2024, TDS deducted on 31-Aug-2024 (26 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (8 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
@@ -2874,7 +2874,7 @@
       <c r="G52" s="2" t="inlineStr"/>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Aug-2024, TDS deducted on 31-Aug-2024 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹4 (392 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 05-Aug-2024, TDS deducted on 31-Aug-2024 (26 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (6 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
@@ -2920,7 +2920,7 @@
       <c r="G53" s="2" t="inlineStr"/>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 10-Sep-2024, TDS deducted on 30-Sep-2024 (20 days late, 1 month(s)). Interest u/s 201(1A): ₹2 (246 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 16-Aug-2024, TDS deducted on 31-Aug-2024 (15 days late, 1 month(s)). Interest u/s 201(1A): ₹2 (205 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
@@ -2966,7 +2966,7 @@
       <c r="G54" s="2" t="inlineStr"/>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 24-Sep-2024, TDS deducted on 30-Sep-2024 (6 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (14 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 16-Aug-2024, TDS deducted on 31-Aug-2024 (15 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (28 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
@@ -3012,7 +3012,7 @@
       <c r="G55" s="2" t="inlineStr"/>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 24-Sep-2024, TDS deducted on 30-Sep-2024 (6 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (12 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 16-Aug-2024, TDS deducted on 31-Aug-2024 (15 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (11 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
@@ -3058,7 +3058,7 @@
       <c r="G56" s="2" t="inlineStr"/>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 07-Oct-2024, TDS deducted on 31-Oct-2024 (24 days late, 1 month(s)). Interest u/s 201(1A): ₹8 (773 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Aug-2024, TDS deducted on 31-Aug-2024 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹4 (392 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
@@ -3104,7 +3104,7 @@
       <c r="G57" s="2" t="inlineStr"/>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 07-Oct-2024, TDS deducted on 31-Oct-2024 (24 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (32 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 10-Sep-2024, TDS deducted on 30-Sep-2024 (20 days late, 1 month(s)). Interest u/s 201(1A): ₹2 (246 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
@@ -3150,7 +3150,7 @@
       <c r="G58" s="2" t="inlineStr"/>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 07-Oct-2024, TDS deducted on 31-Oct-2024 (24 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (18 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 24-Sep-2024, TDS deducted on 30-Sep-2024 (6 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (14 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
@@ -3196,7 +3196,7 @@
       <c r="G59" s="2" t="inlineStr"/>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 19-Oct-2024, TDS deducted on 31-Oct-2024 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (15 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 24-Sep-2024, TDS deducted on 30-Sep-2024 (6 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (12 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
@@ -3242,7 +3242,7 @@
       <c r="G60" s="2" t="inlineStr"/>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 19-Oct-2024, TDS deducted on 31-Oct-2024 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (18 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 07-Oct-2024, TDS deducted on 31-Oct-2024 (24 days late, 1 month(s)). Interest u/s 201(1A): ₹8 (773 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
@@ -3288,7 +3288,7 @@
       <c r="G61" s="2" t="inlineStr"/>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 02-Nov-2024, TDS deducted on 30-Nov-2024 (28 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (6 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 07-Oct-2024, TDS deducted on 31-Oct-2024 (24 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (32 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
@@ -3334,7 +3334,7 @@
       <c r="G62" s="2" t="inlineStr"/>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 02-Nov-2024, TDS deducted on 30-Nov-2024 (28 days late, 1 month(s)). Interest u/s 201(1A): ₹1 (136 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 07-Oct-2024, TDS deducted on 31-Oct-2024 (24 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (18 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
@@ -3380,7 +3380,7 @@
       <c r="G63" s="2" t="inlineStr"/>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 02-Nov-2024, TDS deducted on 30-Nov-2024 (28 days late, 1 month(s)). Interest u/s 201(1A): ₹2 (180 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 19-Oct-2024, TDS deducted on 31-Oct-2024 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (15 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
@@ -3426,7 +3426,7 @@
       <c r="G64" s="2" t="inlineStr"/>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 02-Nov-2024, TDS deducted on 30-Nov-2024 (28 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (12 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 19-Oct-2024, TDS deducted on 31-Oct-2024 (12 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (18 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
@@ -3472,7 +3472,7 @@
       <c r="G65" s="2" t="inlineStr"/>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 12-Nov-2024, TDS deducted on 30-Nov-2024 (18 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (46 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 02-Nov-2024, TDS deducted on 30-Nov-2024 (28 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (6 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
@@ -3518,7 +3518,7 @@
       <c r="G66" s="2" t="inlineStr"/>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 26-Nov-2024, TDS deducted on 30-Nov-2024 (4 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (12 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 02-Nov-2024, TDS deducted on 30-Nov-2024 (28 days late, 1 month(s)). Interest u/s 201(1A): ₹1 (136 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
@@ -3564,7 +3564,7 @@
       <c r="G67" s="2" t="inlineStr"/>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 26-Nov-2024, TDS deducted on 30-Nov-2024 (4 days late, 1 month(s)). Interest u/s 201(1A): ₹1 (74 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 02-Nov-2024, TDS deducted on 30-Nov-2024 (28 days late, 1 month(s)). Interest u/s 201(1A): ₹2 (180 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
@@ -3610,7 +3610,7 @@
       <c r="G68" s="2" t="inlineStr"/>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 26-Nov-2024, TDS deducted on 30-Nov-2024 (4 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (43 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 02-Nov-2024, TDS deducted on 30-Nov-2024 (28 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (12 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
@@ -3656,7 +3656,7 @@
       <c r="G69" s="2" t="inlineStr"/>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 26-Nov-2024, TDS deducted on 30-Nov-2024 (4 days late, 1 month(s)). Interest u/s 201(1A): ₹1 (55 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 12-Nov-2024, TDS deducted on 30-Nov-2024 (18 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (46 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr">
@@ -3702,7 +3702,7 @@
       <c r="G70" s="2" t="inlineStr"/>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 26-Nov-2024, TDS deducted on 30-Nov-2024 (4 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (41 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 26-Nov-2024, TDS deducted on 30-Nov-2024 (4 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (12 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
@@ -3748,7 +3748,7 @@
       <c r="G71" s="2" t="inlineStr"/>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 26-Nov-2024, TDS deducted on 30-Nov-2024 (4 days late, 1 month(s)). Interest u/s 201(1A): ₹1 (118 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 26-Nov-2024, TDS deducted on 30-Nov-2024 (4 days late, 1 month(s)). Interest u/s 201(1A): ₹1 (74 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr">
@@ -3794,7 +3794,7 @@
       <c r="G72" s="2" t="inlineStr"/>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 26-Nov-2024, TDS deducted on 30-Nov-2024 (4 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (42 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 26-Nov-2024, TDS deducted on 30-Nov-2024 (4 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (43 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
@@ -3840,7 +3840,7 @@
       <c r="G73" s="2" t="inlineStr"/>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 26-Nov-2024, TDS deducted on 30-Nov-2024 (4 days late, 1 month(s)). Interest u/s 201(1A): ₹2 (156 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 26-Nov-2024, TDS deducted on 30-Nov-2024 (4 days late, 1 month(s)). Interest u/s 201(1A): ₹1 (55 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr">
@@ -3886,7 +3886,7 @@
       <c r="G74" s="2" t="inlineStr"/>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 26-Nov-2024, TDS deducted on 30-Nov-2024 (4 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (27 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 26-Nov-2024, TDS deducted on 30-Nov-2024 (4 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (41 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
@@ -3932,7 +3932,7 @@
       <c r="G75" s="2" t="inlineStr"/>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Dec-2024, TDS deducted on 31-Dec-2024 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (47 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 26-Nov-2024, TDS deducted on 30-Nov-2024 (4 days late, 1 month(s)). Interest u/s 201(1A): ₹1 (118 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr">
@@ -3978,7 +3978,7 @@
       <c r="G76" s="2" t="inlineStr"/>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Dec-2024, TDS deducted on 31-Dec-2024 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (16 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 26-Nov-2024, TDS deducted on 30-Nov-2024 (4 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (42 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
@@ -4024,7 +4024,7 @@
       <c r="G77" s="2" t="inlineStr"/>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Dec-2024, TDS deducted on 31-Dec-2024 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹1 (61 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 26-Nov-2024, TDS deducted on 30-Nov-2024 (4 days late, 1 month(s)). Interest u/s 201(1A): ₹2 (156 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
@@ -4070,7 +4070,7 @@
       <c r="G78" s="2" t="inlineStr"/>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Dec-2024, TDS deducted on 31-Dec-2024 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹1 (74 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 26-Nov-2024, TDS deducted on 30-Nov-2024 (4 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (27 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
@@ -4116,7 +4116,7 @@
       <c r="G79" s="2" t="inlineStr"/>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Dec-2024, TDS deducted on 31-Dec-2024 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹1 (74 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Dec-2024, TDS deducted on 31-Dec-2024 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (47 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I79" s="2" t="inlineStr">
@@ -4162,7 +4162,7 @@
       <c r="G80" s="2" t="inlineStr"/>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Dec-2024, TDS deducted on 31-Dec-2024 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (28 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Dec-2024, TDS deducted on 31-Dec-2024 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (16 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
@@ -4208,7 +4208,7 @@
       <c r="G81" s="2" t="inlineStr"/>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Dec-2024, TDS deducted on 31-Dec-2024 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (44 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Dec-2024, TDS deducted on 31-Dec-2024 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹1 (61 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I81" s="2" t="inlineStr">
@@ -4254,7 +4254,7 @@
       <c r="G82" s="2" t="inlineStr"/>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Dec-2024, TDS deducted on 31-Dec-2024 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (44 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Dec-2024, TDS deducted on 31-Dec-2024 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹1 (74 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
@@ -4300,7 +4300,7 @@
       <c r="G83" s="2" t="inlineStr"/>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Dec-2024, TDS deducted on 31-Dec-2024 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (28 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Dec-2024, TDS deducted on 31-Dec-2024 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹1 (74 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I83" s="2" t="inlineStr">
@@ -4346,7 +4346,7 @@
       <c r="G84" s="2" t="inlineStr"/>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Dec-2024, TDS deducted on 31-Dec-2024 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (45 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Dec-2024, TDS deducted on 31-Dec-2024 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (28 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
@@ -4392,7 +4392,7 @@
       <c r="G85" s="2" t="inlineStr"/>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Dec-2024, TDS deducted on 31-Dec-2024 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (6 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Dec-2024, TDS deducted on 31-Dec-2024 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (44 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I85" s="2" t="inlineStr">
@@ -4438,7 +4438,7 @@
       <c r="G86" s="2" t="inlineStr"/>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 26-Dec-2024, TDS deducted on 31-Dec-2024 (5 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (31 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Dec-2024, TDS deducted on 31-Dec-2024 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (44 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
@@ -4484,7 +4484,7 @@
       <c r="G87" s="2" t="inlineStr"/>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 26-Dec-2024, TDS deducted on 31-Dec-2024 (5 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (41 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Dec-2024, TDS deducted on 31-Dec-2024 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (28 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I87" s="2" t="inlineStr">
@@ -4530,7 +4530,7 @@
       <c r="G88" s="2" t="inlineStr"/>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 26-Dec-2024, TDS deducted on 31-Dec-2024 (5 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (12 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Dec-2024, TDS deducted on 31-Dec-2024 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (45 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr">
@@ -4576,7 +4576,7 @@
       <c r="G89" s="2" t="inlineStr"/>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 10-Jan-2025, TDS deducted on 31-Jan-2025 (21 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (43 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Dec-2024, TDS deducted on 31-Dec-2024 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (6 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I89" s="2" t="inlineStr">
@@ -4622,7 +4622,7 @@
       <c r="G90" s="2" t="inlineStr"/>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 10-Jan-2025, TDS deducted on 31-Jan-2025 (21 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (47 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 26-Dec-2024, TDS deducted on 31-Dec-2024 (5 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (31 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       <c r="G91" s="2" t="inlineStr"/>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 10-Jan-2025, TDS deducted on 31-Jan-2025 (21 days late, 1 month(s)). Interest u/s 201(1A): ₹1 (106 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 26-Dec-2024, TDS deducted on 31-Dec-2024 (5 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (41 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr">
@@ -4714,7 +4714,7 @@
       <c r="G92" s="2" t="inlineStr"/>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 07-Feb-2025, TDS deducted on 28-Feb-2025 (21 days late, 1 month(s)). Interest u/s 201(1A): ₹3 (319 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 26-Dec-2024, TDS deducted on 31-Dec-2024 (5 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (12 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr">
@@ -4760,7 +4760,7 @@
       <c r="G93" s="2" t="inlineStr"/>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 07-Feb-2025, TDS deducted on 28-Feb-2025 (21 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (47 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 10-Jan-2025, TDS deducted on 31-Jan-2025 (21 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (43 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I93" s="2" t="inlineStr">
@@ -4806,7 +4806,7 @@
       <c r="G94" s="2" t="inlineStr"/>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 07-Feb-2025, TDS deducted on 28-Feb-2025 (21 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (11 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 10-Jan-2025, TDS deducted on 31-Jan-2025 (21 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (47 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I94" s="2" t="inlineStr">
@@ -4852,7 +4852,7 @@
       <c r="G95" s="2" t="inlineStr"/>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Mar-2025, TDS deducted on 31-Mar-2025 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (19 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 10-Jan-2025, TDS deducted on 31-Jan-2025 (21 days late, 1 month(s)). Interest u/s 201(1A): ₹1 (106 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I95" s="2" t="inlineStr">
@@ -4882,23 +4882,23 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>SAHIB S CHOUDHARY &amp; COMPANY</t>
+          <t>INLAND WORLD LOGISTICS PVT LTD</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>AEJPC0634D</t>
+          <t>AAACI5607C</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>194J(b)</t>
+          <t>194C</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr"/>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on SAHIB S CHOUDHARY &amp; COMPANY (194J(b)): Expense on 07-Jan-2025, TDS deducted on 31-Jan-2025 (24 days late, 1 month(s)). Interest u/s 201(1A): ₹9 (900 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 07-Feb-2025, TDS deducted on 28-Feb-2025 (21 days late, 1 month(s)). Interest u/s 201(1A): ₹3 (319 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I96" s="2" t="inlineStr">
@@ -4928,23 +4928,23 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>SNCL BUILDERS LLP</t>
+          <t>INLAND WORLD LOGISTICS PVT LTD</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>ADXFS1033K</t>
+          <t>AAACI5607C</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>194J(b)</t>
+          <t>194C</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr"/>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on SNCL BUILDERS LLP (194J(b)): Expense on 05-Dec-2024, TDS deducted on 31-Dec-2024 (26 days late, 1 month(s)). Interest u/s 201(1A): ₹120 (12,000 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 07-Feb-2025, TDS deducted on 28-Feb-2025 (21 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (47 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I97" s="2" t="inlineStr">
@@ -4974,23 +4974,23 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>GST PROFESSIONALS LLP</t>
+          <t>INLAND WORLD LOGISTICS PVT LTD</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>AAPFG3370E</t>
+          <t>AAACI5607C</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>194J(b)</t>
+          <t>194C</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr"/>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on GST PROFESSIONALS LLP (194J(b)): Expense on 30-Nov-2024, TDS deducted on 31-Dec-2024 (31 days late, 2 month(s)). Interest u/s 201(1A): ₹30 (1,500 × 1% × 2 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 07-Feb-2025, TDS deducted on 28-Feb-2025 (21 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (11 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I98" s="2" t="inlineStr">
@@ -5020,23 +5020,23 @@
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>GST PROFESSIONALS LLP</t>
+          <t>INLAND WORLD LOGISTICS PVT LTD</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>AAPFG3370E</t>
+          <t>AAACI5607C</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>194J(b)</t>
+          <t>194C</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr"/>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on GST PROFESSIONALS LLP (194J(b)): Expense on 24-Dec-2024, TDS deducted on 31-Dec-2024 (7 days late, 1 month(s)). Interest u/s 201(1A): ₹16 (1,650 × 1% × 1 months).</t>
+          <t>Late TDS deduction on INLAND WORLD LOGISTICS PVT LTD (194C): Expense on 17-Mar-2025, TDS deducted on 31-Mar-2025 (14 days late, 1 month(s)). Interest u/s 201(1A): ₹0 (19 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I99" s="2" t="inlineStr">
@@ -5066,23 +5066,23 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>RAYMOND LIFESTYLE LTD.</t>
+          <t>SAHIB S CHOUDHARY &amp; COMPANY</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>AAJCR2207E</t>
+          <t>AEJPC0634D</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>194Q</t>
+          <t>194J(b)</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr"/>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on RAYMOND LIFESTYLE LTD. (194Q): Expense on 28-Dec-2024, TDS deducted on 31-Dec-2024 (3 days late, 1 month(s)). Interest u/s 201(1A): ₹138 (13,796 × 1% × 1 months).</t>
+          <t>Late TDS deduction on SAHIB S CHOUDHARY &amp; COMPANY (194J(b)): Expense on 07-Jan-2025, TDS deducted on 31-Jan-2025 (24 days late, 1 month(s)). Interest u/s 201(1A): ₹9 (900 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I100" s="2" t="inlineStr">
@@ -5112,23 +5112,23 @@
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>RAYMOND LIFESTYLE LTD.</t>
+          <t>SNCL BUILDERS LLP</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>AAJCR2207E</t>
+          <t>ADXFS1033K</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>194Q</t>
+          <t>194J(b)</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr"/>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on RAYMOND LIFESTYLE LTD. (194Q): Expense on 28-Mar-2025, TDS deducted on 31-Mar-2025 (3 days late, 1 month(s)). Interest u/s 201(1A): ₹79 (7,935 × 1% × 1 months).</t>
+          <t>Late TDS deduction on SNCL BUILDERS LLP (194J(b)): Expense on 05-Dec-2024, TDS deducted on 31-Dec-2024 (26 days late, 1 month(s)). Interest u/s 201(1A): ₹120 (12,000 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I101" s="2" t="inlineStr">
@@ -5158,23 +5158,23 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>Raymond Limited</t>
+          <t>GST PROFESSIONALS LLP</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>AAACR4896A</t>
+          <t>AAPFG3370E</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>194Q</t>
+          <t>194J(b)</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr"/>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on Raymond Limited (194Q): Expense on 28-Jun-2024, TDS deducted on 30-Jun-2024 (2 days late, 1 month(s)). Interest u/s 201(1A): ₹15 (1,481 × 1% × 1 months).</t>
+          <t>Late TDS deduction on GST PROFESSIONALS LLP (194J(b)): Expense on 30-Nov-2024, TDS deducted on 31-Dec-2024 (31 days late, 2 month(s)). Interest u/s 201(1A): ₹30 (1,500 × 1% × 2 months).</t>
         </is>
       </c>
       <c r="I102" s="2" t="inlineStr">
@@ -5204,23 +5204,23 @@
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>Sai Boutique</t>
+          <t>GST PROFESSIONALS LLP</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>AEPFS3230M</t>
+          <t>AAPFG3370E</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>194Q</t>
+          <t>194J(b)</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr"/>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on Sai Boutique (194Q): Expense on 28-Jan-2025, TDS deducted on 31-Jan-2025 (3 days late, 1 month(s)). Interest u/s 201(1A): ₹4 (382 × 1% × 1 months).</t>
+          <t>Late TDS deduction on GST PROFESSIONALS LLP (194J(b)): Expense on 24-Dec-2024, TDS deducted on 31-Dec-2024 (7 days late, 1 month(s)). Interest u/s 201(1A): ₹16 (1,650 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I103" s="2" t="inlineStr">
@@ -5266,7 +5266,7 @@
       <c r="G104" s="2" t="inlineStr"/>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on RAYMOND LIFESTYLE LTD. (194Q): Expense on 28-Sep-2024, TDS deducted on 30-Sep-2024 (2 days late, 1 month(s)). Interest u/s 201(1A): ₹145 (14,544 × 1% × 1 months).</t>
+          <t>Late TDS deduction on RAYMOND LIFESTYLE LTD. (194Q): Expense on 28-Dec-2024, TDS deducted on 31-Dec-2024 (3 days late, 1 month(s)). Interest u/s 201(1A): ₹138 (13,796 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I104" s="2" t="inlineStr">
@@ -5312,7 +5312,7 @@
       <c r="G105" s="2" t="inlineStr"/>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>Late TDS deduction on RAYMOND LIFESTYLE LTD. (194Q): Expense on 28-Oct-2024, TDS deducted on 31-Oct-2024 (3 days late, 1 month(s)). Interest u/s 201(1A): ₹25 (2,463 × 1% × 1 months).</t>
+          <t>Late TDS deduction on RAYMOND LIFESTYLE LTD. (194Q): Expense on 28-Mar-2025, TDS deducted on 31-Mar-2025 (3 days late, 1 month(s)). Interest u/s 201(1A): ₹79 (7,935 × 1% × 1 months).</t>
         </is>
       </c>
       <c r="I105" s="2" t="inlineStr">
@@ -5342,12 +5342,12 @@
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>RAYMOND LIFESTYLE LTD.</t>
+          <t>Raymond Limited</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>AAJCR2207E</t>
+          <t>AAACR4896A</t>
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr">
@@ -5358,199 +5358,199 @@
       <c r="G106" s="2" t="inlineStr"/>
       <c r="H106" s="2" t="inlineStr">
         <is>
+          <t>Late TDS deduction on Raymond Limited (194Q): Expense on 28-Jun-2024, TDS deducted on 30-Jun-2024 (2 days late, 1 month(s)). Interest u/s 201(1A): ₹15 (1,481 × 1% × 1 months).</t>
+        </is>
+      </c>
+      <c r="I106" s="2" t="inlineStr">
+        <is>
+          <t>Manual review required.</t>
+        </is>
+      </c>
+      <c r="J106" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>tds_timing</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>Sai Boutique</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>AEPFS3230M</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>194Q</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr"/>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
+          <t>Late TDS deduction on Sai Boutique (194Q): Expense on 28-Jan-2025, TDS deducted on 31-Jan-2025 (3 days late, 1 month(s)). Interest u/s 201(1A): ₹4 (382 × 1% × 1 months).</t>
+        </is>
+      </c>
+      <c r="I107" s="2" t="inlineStr">
+        <is>
+          <t>Manual review required.</t>
+        </is>
+      </c>
+      <c r="J107" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>tds_timing</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>RAYMOND LIFESTYLE LTD.</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>AAJCR2207E</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>194Q</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr"/>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>Late TDS deduction on RAYMOND LIFESTYLE LTD. (194Q): Expense on 28-Sep-2024, TDS deducted on 30-Sep-2024 (2 days late, 1 month(s)). Interest u/s 201(1A): ₹145 (14,544 × 1% × 1 months).</t>
+        </is>
+      </c>
+      <c r="I108" s="2" t="inlineStr">
+        <is>
+          <t>Manual review required.</t>
+        </is>
+      </c>
+      <c r="J108" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>tds_timing</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>RAYMOND LIFESTYLE LTD.</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>AAJCR2207E</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>194Q</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr"/>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>Late TDS deduction on RAYMOND LIFESTYLE LTD. (194Q): Expense on 28-Oct-2024, TDS deducted on 31-Oct-2024 (3 days late, 1 month(s)). Interest u/s 201(1A): ₹25 (2,463 × 1% × 1 months).</t>
+        </is>
+      </c>
+      <c r="I109" s="2" t="inlineStr">
+        <is>
+          <t>Manual review required.</t>
+        </is>
+      </c>
+      <c r="J109" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>tds_timing</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>RAYMOND LIFESTYLE LTD.</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>AAJCR2207E</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>194Q</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr"/>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
           <t>Late TDS deduction on RAYMOND LIFESTYLE LTD. (194Q): Expense on 28-Jan-2025, TDS deducted on 31-Jan-2025 (3 days late, 1 month(s)). Interest u/s 201(1A): ₹59 (5,948 × 1% × 1 months).</t>
         </is>
       </c>
-      <c r="I106" s="2" t="inlineStr">
+      <c r="I110" s="2" t="inlineStr">
         <is>
           <t>Manual review required.</t>
         </is>
       </c>
-      <c r="J106" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="3" t="n">
-        <v>106</v>
-      </c>
-      <c r="B107" s="3" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="C107" s="3" t="inlineStr">
-        <is>
-          <t>section_validation</t>
-        </is>
-      </c>
-      <c r="D107" s="3" t="inlineStr">
-        <is>
-          <t>ANDREAL INNOVATION PVT LTD</t>
-        </is>
-      </c>
-      <c r="E107" s="3" t="inlineStr">
-        <is>
-          <t>ABACA2255R</t>
-        </is>
-      </c>
-      <c r="F107" s="3" t="inlineStr">
-        <is>
-          <t>194C</t>
-        </is>
-      </c>
-      <c r="G107" s="3" t="inlineStr"/>
-      <c r="H107" s="3" t="inlineStr">
-        <is>
-          <t>Ambiguous expense(s): Advertisement. Section 194C is possible but verify against invoice/contract nature.</t>
-        </is>
-      </c>
-      <c r="I107" s="3" t="inlineStr">
-        <is>
-          <t>Ambiguous classification — verify invoice nature. If advertisement is creative/professional service → 194J(b). If it's production/printing contract work → 194C. Obtain vendor declaration if uncertain.</t>
-        </is>
-      </c>
-      <c r="J107" s="3" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="3" t="n">
-        <v>107</v>
-      </c>
-      <c r="B108" s="3" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="C108" s="3" t="inlineStr">
-        <is>
-          <t>section_validation</t>
-        </is>
-      </c>
-      <c r="D108" s="3" t="inlineStr">
-        <is>
-          <t>ANDERSON TECHNOLOGY PVT LTD</t>
-        </is>
-      </c>
-      <c r="E108" s="3" t="inlineStr">
-        <is>
-          <t>AAFCA4805K</t>
-        </is>
-      </c>
-      <c r="F108" s="3" t="inlineStr">
-        <is>
-          <t>194C</t>
-        </is>
-      </c>
-      <c r="G108" s="3" t="inlineStr"/>
-      <c r="H108" s="3" t="inlineStr">
-        <is>
-          <t>Ambiguous expense(s): Advertisement. Section 194C is possible but verify against invoice/contract nature.</t>
-        </is>
-      </c>
-      <c r="I108" s="3" t="inlineStr">
-        <is>
-          <t>Ambiguous classification — verify invoice nature. If advertisement is creative/professional service → 194J(b). If it's production/printing contract work → 194C. Obtain vendor declaration if uncertain.</t>
-        </is>
-      </c>
-      <c r="J108" s="3" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="3" t="n">
-        <v>108</v>
-      </c>
-      <c r="B109" s="3" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="C109" s="3" t="inlineStr">
-        <is>
-          <t>section_validation</t>
-        </is>
-      </c>
-      <c r="D109" s="3" t="inlineStr">
-        <is>
-          <t>ANDERSON TECHNOLOGY PVT LTD</t>
-        </is>
-      </c>
-      <c r="E109" s="3" t="inlineStr">
-        <is>
-          <t>AAFCA4805K</t>
-        </is>
-      </c>
-      <c r="F109" s="3" t="inlineStr">
-        <is>
-          <t>194C</t>
-        </is>
-      </c>
-      <c r="G109" s="3" t="inlineStr"/>
-      <c r="H109" s="3" t="inlineStr">
-        <is>
-          <t>Ambiguous expense(s): Advertisement. Section 194C is possible but verify against invoice/contract nature.</t>
-        </is>
-      </c>
-      <c r="I109" s="3" t="inlineStr">
-        <is>
-          <t>Ambiguous classification — verify invoice nature. If advertisement is creative/professional service → 194J(b). If it's production/printing contract work → 194C. Obtain vendor declaration if uncertain.</t>
-        </is>
-      </c>
-      <c r="J109" s="3" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="3" t="n">
-        <v>109</v>
-      </c>
-      <c r="B110" s="3" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="C110" s="3" t="inlineStr">
-        <is>
-          <t>section_validation</t>
-        </is>
-      </c>
-      <c r="D110" s="3" t="inlineStr">
-        <is>
-          <t>ANDERSON TECHNOLOGY PVT LTD</t>
-        </is>
-      </c>
-      <c r="E110" s="3" t="inlineStr">
-        <is>
-          <t>AAFCA4805K</t>
-        </is>
-      </c>
-      <c r="F110" s="3" t="inlineStr">
-        <is>
-          <t>194C</t>
-        </is>
-      </c>
-      <c r="G110" s="3" t="inlineStr"/>
-      <c r="H110" s="3" t="inlineStr">
-        <is>
-          <t>Ambiguous expense(s): Advertisement. Section 194C is possible but verify against invoice/contract nature.</t>
-        </is>
-      </c>
-      <c r="I110" s="3" t="inlineStr">
-        <is>
-          <t>Ambiguous classification — verify invoice nature. If advertisement is creative/professional service → 194J(b). If it's production/printing contract work → 194C. Obtain vendor declaration if uncertain.</t>
-        </is>
-      </c>
-      <c r="J110" s="3" t="inlineStr">
+      <c r="J110" s="2" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -5613,31 +5613,33 @@
       </c>
       <c r="C112" s="3" t="inlineStr">
         <is>
-          <t>missing_tds</t>
+          <t>section_validation</t>
         </is>
       </c>
       <c r="D112" s="3" t="inlineStr">
         <is>
-          <t>Kochar Tradelink LLP</t>
-        </is>
-      </c>
-      <c r="E112" s="3" t="inlineStr"/>
+          <t>ANDERSON TECHNOLOGY PVT LTD</t>
+        </is>
+      </c>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>AAFCA4805K</t>
+        </is>
+      </c>
       <c r="F112" s="3" t="inlineStr">
         <is>
-          <t>194H</t>
-        </is>
-      </c>
-      <c r="G112" s="3" t="n">
-        <v>44932</v>
-      </c>
+          <t>194C</t>
+        </is>
+      </c>
+      <c r="G112" s="3" t="inlineStr"/>
       <c r="H112" s="3" t="inlineStr">
         <is>
-          <t>No Form 26 entry found for Kochar Tradelink LLP under 194H. Tally shows ₹44,932 in Brokerage and Commission. TDS may be missing. Review: Has entries on quarter/year-end dates (2025-03-31) alongside other dates — may include provisions or reversals. | Same transaction (₹38,743) appears in both Journal Register and GST Exp Register — counted once from Journal. Please confirm these are the same entry.</t>
+          <t>Ambiguous expense(s): Advertisement. Section 194C is possible but verify against invoice/contract nature.</t>
         </is>
       </c>
       <c r="I112" s="3" t="inlineStr">
         <is>
-          <t>Tally shows expenses to this vendor but no TDS was deducted in Form 26. Action required: (1) Check if vendor provided Form 15G/15H or lower deduction certificate. (2) If not, deduct TDS immediately and deposit with interest u/s 201(1A) at 1% per month. (3) File revised TDS return for the applicable quarter.</t>
+          <t>Ambiguous classification — verify invoice nature. If advertisement is creative/professional service → 194J(b). If it's production/printing contract work → 194C. Obtain vendor declaration if uncertain.</t>
         </is>
       </c>
       <c r="J112" s="3" t="inlineStr">
@@ -5657,231 +5659,413 @@
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
+          <t>section_validation</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>ANDERSON TECHNOLOGY PVT LTD</t>
+        </is>
+      </c>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t>AAFCA4805K</t>
+        </is>
+      </c>
+      <c r="F113" s="3" t="inlineStr">
+        <is>
+          <t>194C</t>
+        </is>
+      </c>
+      <c r="G113" s="3" t="inlineStr"/>
+      <c r="H113" s="3" t="inlineStr">
+        <is>
+          <t>Ambiguous expense(s): Advertisement. Section 194C is possible but verify against invoice/contract nature.</t>
+        </is>
+      </c>
+      <c r="I113" s="3" t="inlineStr">
+        <is>
+          <t>Ambiguous classification — verify invoice nature. If advertisement is creative/professional service → 194J(b). If it's production/printing contract work → 194C. Obtain vendor declaration if uncertain.</t>
+        </is>
+      </c>
+      <c r="J113" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="3" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>section_validation</t>
+        </is>
+      </c>
+      <c r="D114" s="3" t="inlineStr">
+        <is>
+          <t>ANDERSON TECHNOLOGY PVT LTD</t>
+        </is>
+      </c>
+      <c r="E114" s="3" t="inlineStr">
+        <is>
+          <t>AAFCA4805K</t>
+        </is>
+      </c>
+      <c r="F114" s="3" t="inlineStr">
+        <is>
+          <t>194C</t>
+        </is>
+      </c>
+      <c r="G114" s="3" t="inlineStr"/>
+      <c r="H114" s="3" t="inlineStr">
+        <is>
+          <t>Ambiguous expense(s): Advertisement. Section 194C is possible but verify against invoice/contract nature.</t>
+        </is>
+      </c>
+      <c r="I114" s="3" t="inlineStr">
+        <is>
+          <t>Ambiguous classification — verify invoice nature. If advertisement is creative/professional service → 194J(b). If it's production/printing contract work → 194C. Obtain vendor declaration if uncertain.</t>
+        </is>
+      </c>
+      <c r="J114" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="3" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" s="3" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="inlineStr">
+        <is>
+          <t>section_validation</t>
+        </is>
+      </c>
+      <c r="D115" s="3" t="inlineStr">
+        <is>
+          <t>ANDREAL INNOVATION PVT LTD</t>
+        </is>
+      </c>
+      <c r="E115" s="3" t="inlineStr">
+        <is>
+          <t>ABACA2255R</t>
+        </is>
+      </c>
+      <c r="F115" s="3" t="inlineStr">
+        <is>
+          <t>194C</t>
+        </is>
+      </c>
+      <c r="G115" s="3" t="inlineStr"/>
+      <c r="H115" s="3" t="inlineStr">
+        <is>
+          <t>Ambiguous expense(s): Advertisement. Section 194C is possible but verify against invoice/contract nature.</t>
+        </is>
+      </c>
+      <c r="I115" s="3" t="inlineStr">
+        <is>
+          <t>Ambiguous classification — verify invoice nature. If advertisement is creative/professional service → 194J(b). If it's production/printing contract work → 194C. Obtain vendor declaration if uncertain.</t>
+        </is>
+      </c>
+      <c r="J115" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="3" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" s="3" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
           <t>missing_tds</t>
         </is>
       </c>
-      <c r="D113" s="3" t="inlineStr">
+      <c r="D116" s="3" t="inlineStr">
+        <is>
+          <t>Kochar Tradelink LLP</t>
+        </is>
+      </c>
+      <c r="E116" s="3" t="inlineStr"/>
+      <c r="F116" s="3" t="inlineStr">
+        <is>
+          <t>194H</t>
+        </is>
+      </c>
+      <c r="G116" s="3" t="n">
+        <v>44932</v>
+      </c>
+      <c r="H116" s="3" t="inlineStr">
+        <is>
+          <t>No Form 26 entry found for Kochar Tradelink LLP under 194H. Tally shows ₹44,932 in Brokerage and Commission. TDS may be missing. Review: Has entries on quarter/year-end dates (2025-03-31) alongside other dates — may include provisions or reversals. | Same transaction (₹38,743) appears in both Journal Register and GST Exp Register — counted once from Journal. Please confirm these are the same entry.</t>
+        </is>
+      </c>
+      <c r="I116" s="3" t="inlineStr">
+        <is>
+          <t>Tally shows expenses to this vendor but no TDS was deducted in Form 26. Action required: (1) Check if vendor provided Form 15G/15H or lower deduction certificate. (2) If not, deduct TDS immediately and deposit with interest u/s 201(1A) at 1% per month. (3) File revised TDS return for the applicable quarter.</t>
+        </is>
+      </c>
+      <c r="J116" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="3" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" s="3" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>missing_tds</t>
+        </is>
+      </c>
+      <c r="D117" s="3" t="inlineStr">
         <is>
           <t>Pukesh Sharma</t>
         </is>
       </c>
-      <c r="E113" s="3" t="inlineStr"/>
-      <c r="F113" s="3" t="inlineStr">
+      <c r="E117" s="3" t="inlineStr"/>
+      <c r="F117" s="3" t="inlineStr">
         <is>
           <t>194H</t>
         </is>
       </c>
-      <c r="G113" s="3" t="n">
+      <c r="G117" s="3" t="n">
         <v>20877</v>
       </c>
-      <c r="H113" s="3" t="inlineStr">
+      <c r="H117" s="3" t="inlineStr">
         <is>
           <t>No Form 26 entry found for Pukesh Sharma under 194H. Tally shows ₹20,877 in Brokerage and Commission. TDS may be missing. Review: Has entries on quarter/year-end dates (2025-03-31) alongside other dates — may include provisions or reversals.</t>
         </is>
       </c>
-      <c r="I113" s="3" t="inlineStr">
+      <c r="I117" s="3" t="inlineStr">
         <is>
           <t>Tally shows expenses to this vendor but no TDS was deducted in Form 26. Action required: (1) Check if vendor provided Form 15G/15H or lower deduction certificate. (2) If not, deduct TDS immediately and deposit with interest u/s 201(1A) at 1% per month. (3) File revised TDS return for the applicable quarter.</t>
         </is>
       </c>
-      <c r="J113" s="3" t="inlineStr">
+      <c r="J117" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" s="4" t="n">
-        <v>113</v>
-      </c>
-      <c r="B114" s="4" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="4" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" s="4" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="C114" s="4" t="inlineStr">
+      <c r="C118" s="4" t="inlineStr">
         <is>
           <t>section_validation</t>
         </is>
       </c>
-      <c r="D114" s="4" t="inlineStr">
+      <c r="D118" s="4" t="inlineStr">
         <is>
           <t>GST PROFESSIONALS LLP</t>
         </is>
       </c>
-      <c r="E114" s="4" t="inlineStr">
+      <c r="E118" s="4" t="inlineStr">
         <is>
           <t>AAPFG3370E</t>
         </is>
       </c>
-      <c r="F114" s="4" t="inlineStr">
+      <c r="F118" s="4" t="inlineStr">
         <is>
           <t>194J(b)</t>
         </is>
       </c>
-      <c r="G114" s="4" t="inlineStr"/>
-      <c r="H114" s="4" t="inlineStr">
+      <c r="G118" s="4" t="inlineStr"/>
+      <c r="H118" s="4" t="inlineStr">
         <is>
           <t>Cannot classify expense(s): Professonal Charges. Manual review needed.</t>
         </is>
       </c>
-      <c r="I114" s="4" t="inlineStr">
+      <c r="I118" s="4" t="inlineStr">
         <is>
           <t>Expense head could not be auto-classified. Manually review the vendor invoice and assign the correct TDS section.</t>
         </is>
       </c>
-      <c r="J114" s="4" t="inlineStr">
+      <c r="J118" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" s="4" t="n">
-        <v>114</v>
-      </c>
-      <c r="B115" s="4" t="inlineStr">
+    <row r="119">
+      <c r="A119" s="4" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" s="4" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="C115" s="4" t="inlineStr">
+      <c r="C119" s="4" t="inlineStr">
         <is>
           <t>threshold_validation</t>
         </is>
       </c>
-      <c r="D115" s="4" t="inlineStr">
+      <c r="D119" s="4" t="inlineStr">
         <is>
           <t>SAHIB S CHOUDHARY &amp; COMPANY</t>
         </is>
       </c>
-      <c r="E115" s="4" t="inlineStr">
+      <c r="E119" s="4" t="inlineStr">
         <is>
           <t>AEJPC0634D</t>
         </is>
       </c>
-      <c r="F115" s="4" t="inlineStr">
+      <c r="F119" s="4" t="inlineStr">
         <is>
           <t>194J(b)</t>
         </is>
       </c>
-      <c r="G115" s="4" t="n">
+      <c r="G119" s="4" t="n">
         <v>9000</v>
       </c>
-      <c r="H115" s="4" t="inlineStr">
-        <is>
-          <t>194J(b) for SAHIB S CHOUDHARY &amp; COMPANY: aggregate ₹9,000 is below annual threshold ₹30,000. TDS deduction is not mandatory (but not wrong if deducted).</t>
-        </is>
-      </c>
-      <c r="I115" s="4" t="inlineStr">
+      <c r="H119" s="4" t="inlineStr">
+        <is>
+          <t>194J(b) for SAHIB S CHOUDHARY &amp; COMPANY: Form 26 aggregate ₹9,000 is below annual threshold ₹30,000. TDS deduction is voluntary. Note: verify total books expense for this vendor is also below threshold.</t>
+        </is>
+      </c>
+      <c r="I119" s="4" t="inlineStr">
         <is>
           <t>TDS was deducted even though aggregate amount is below the threshold. This is not an error — voluntary TDS deduction is valid. No action needed, but note for internal records.</t>
         </is>
       </c>
-      <c r="J115" s="4" t="inlineStr">
+      <c r="J119" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
-    <row r="116">
-      <c r="A116" s="4" t="n">
-        <v>115</v>
-      </c>
-      <c r="B116" s="4" t="inlineStr">
+    <row r="120">
+      <c r="A120" s="4" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" s="4" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="C116" s="4" t="inlineStr">
+      <c r="C120" s="4" t="inlineStr">
         <is>
           <t>threshold_validation</t>
         </is>
       </c>
-      <c r="D116" s="4" t="inlineStr">
+      <c r="D120" s="4" t="inlineStr">
         <is>
           <t>Raymond Limited</t>
         </is>
       </c>
-      <c r="E116" s="4" t="inlineStr">
+      <c r="E120" s="4" t="inlineStr">
         <is>
           <t>AAACR4896A</t>
         </is>
       </c>
-      <c r="F116" s="4" t="inlineStr">
+      <c r="F120" s="4" t="inlineStr">
         <is>
           <t>194Q</t>
         </is>
       </c>
-      <c r="G116" s="4" t="n">
+      <c r="G120" s="4" t="n">
         <v>1480982</v>
       </c>
-      <c r="H116" s="4" t="inlineStr">
-        <is>
-          <t>194Q for Raymond Limited: aggregate ₹1,480,982 is below annual threshold ₹5,000,000. TDS deduction is not mandatory (but not wrong if deducted).</t>
-        </is>
-      </c>
-      <c r="I116" s="4" t="inlineStr">
+      <c r="H120" s="4" t="inlineStr">
+        <is>
+          <t>194Q for Raymond Limited: Form 26 aggregate ₹1,480,982 is below annual threshold ₹5,000,000. TDS deduction is voluntary. Note: verify total books expense for this vendor is also below threshold.</t>
+        </is>
+      </c>
+      <c r="I120" s="4" t="inlineStr">
         <is>
           <t>TDS was deducted even though aggregate amount is below the threshold. This is not an error — voluntary TDS deduction is valid. No action needed, but note for internal records.</t>
         </is>
       </c>
-      <c r="J116" s="4" t="inlineStr">
+      <c r="J120" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
-    <row r="117">
-      <c r="A117" s="4" t="n">
-        <v>116</v>
-      </c>
-      <c r="B117" s="4" t="inlineStr">
+    <row r="121">
+      <c r="A121" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" s="4" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="C117" s="4" t="inlineStr">
+      <c r="C121" s="4" t="inlineStr">
         <is>
           <t>threshold_validation</t>
         </is>
       </c>
-      <c r="D117" s="4" t="inlineStr">
+      <c r="D121" s="4" t="inlineStr">
         <is>
           <t>Sai Boutique</t>
         </is>
       </c>
-      <c r="E117" s="4" t="inlineStr">
+      <c r="E121" s="4" t="inlineStr">
         <is>
           <t>AEPFS3230M</t>
         </is>
       </c>
-      <c r="F117" s="4" t="inlineStr">
+      <c r="F121" s="4" t="inlineStr">
         <is>
           <t>194Q</t>
         </is>
       </c>
-      <c r="G117" s="4" t="n">
+      <c r="G121" s="4" t="n">
         <v>381820</v>
       </c>
-      <c r="H117" s="4" t="inlineStr">
-        <is>
-          <t>194Q for Sai Boutique: aggregate ₹381,820 is below annual threshold ₹5,000,000. TDS deduction is not mandatory (but not wrong if deducted).</t>
-        </is>
-      </c>
-      <c r="I117" s="4" t="inlineStr">
+      <c r="H121" s="4" t="inlineStr">
+        <is>
+          <t>194Q for Sai Boutique: Form 26 aggregate ₹381,820 is below annual threshold ₹5,000,000. TDS deduction is voluntary. Note: verify total books expense for this vendor is also below threshold.</t>
+        </is>
+      </c>
+      <c r="I121" s="4" t="inlineStr">
         <is>
           <t>TDS was deducted even though aggregate amount is below the threshold. This is not an error — voluntary TDS deduction is valid. No action needed, but note for internal records.</t>
         </is>
       </c>
-      <c r="J117" s="4" t="inlineStr">
+      <c r="J121" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J117"/>
+  <autoFilter ref="A1:J121"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix threshold check: use total books expense, not just Form 26 amount
Simple logic: look up total Tally expenses for vendor in that section.
If books total >= threshold → TDS is mandatory, no below-threshold finding.
If books total < threshold → TDS is voluntary, flag as info.

Sahib: total books = ₹39,000 > ₹30,000 threshold → no longer shows
misleading "TDS not mandatory" finding. partial_tds ERROR remains.

https://claude.ai/code/session_01U1MuRvDgn4XPQ38Fe5qjWF
</commit_message>
<xml_diff>
--- a/tds-recon/data/results/tds_recon_report.xlsx
+++ b/tds-recon/data/results/tds_recon_report.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Late TDS Deposit" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Issues for Review'!$A$1:$J$121</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Issues for Review'!$A$1:$J$128</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'TDS Report - Matched'!$A$1:$Q$80</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Zero TDS - Exempt'!$A$1:$G$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Late TDS Deduction'!$A$1:$N$105</definedName>
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J121"/>
+  <dimension ref="A1:J128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5936,25 +5936,25 @@
       </c>
       <c r="D119" s="4" t="inlineStr">
         <is>
-          <t>SAHIB S CHOUDHARY &amp; COMPANY</t>
+          <t>Adi Debnath</t>
         </is>
       </c>
       <c r="E119" s="4" t="inlineStr">
         <is>
-          <t>AEJPC0634D</t>
+          <t>AAAAA0001A</t>
         </is>
       </c>
       <c r="F119" s="4" t="inlineStr">
         <is>
-          <t>194J(b)</t>
+          <t>194A</t>
         </is>
       </c>
       <c r="G119" s="4" t="n">
-        <v>9000</v>
+        <v>344553</v>
       </c>
       <c r="H119" s="4" t="inlineStr">
         <is>
-          <t>194J(b) for SAHIB S CHOUDHARY &amp; COMPANY: Form 26 aggregate ₹9,000 is below annual threshold ₹30,000. TDS deduction is voluntary. Note: verify total books expense for this vendor is also below threshold.</t>
+          <t>194A for Adi Debnath: total expenses in books ₹0 is below annual threshold ₹5,000. TDS deduction is voluntary (not wrong if deducted).</t>
         </is>
       </c>
       <c r="I119" s="4" t="inlineStr">
@@ -5984,25 +5984,25 @@
       </c>
       <c r="D120" s="4" t="inlineStr">
         <is>
-          <t>Raymond Limited</t>
+          <t>Asha Negi</t>
         </is>
       </c>
       <c r="E120" s="4" t="inlineStr">
         <is>
-          <t>AAACR4896A</t>
+          <t>AAAAA0002A</t>
         </is>
       </c>
       <c r="F120" s="4" t="inlineStr">
         <is>
-          <t>194Q</t>
+          <t>194A</t>
         </is>
       </c>
       <c r="G120" s="4" t="n">
-        <v>1480982</v>
+        <v>519695</v>
       </c>
       <c r="H120" s="4" t="inlineStr">
         <is>
-          <t>194Q for Raymond Limited: Form 26 aggregate ₹1,480,982 is below annual threshold ₹5,000,000. TDS deduction is voluntary. Note: verify total books expense for this vendor is also below threshold.</t>
+          <t>194A for Asha Negi: total expenses in books ₹0 is below annual threshold ₹5,000. TDS deduction is voluntary (not wrong if deducted).</t>
         </is>
       </c>
       <c r="I120" s="4" t="inlineStr">
@@ -6032,40 +6032,376 @@
       </c>
       <c r="D121" s="4" t="inlineStr">
         <is>
-          <t>Sai Boutique</t>
+          <t>Manisha Kumari</t>
         </is>
       </c>
       <c r="E121" s="4" t="inlineStr">
         <is>
-          <t>AEPFS3230M</t>
+          <t>AAAAA0003A</t>
         </is>
       </c>
       <c r="F121" s="4" t="inlineStr">
         <is>
+          <t>194A</t>
+        </is>
+      </c>
+      <c r="G121" s="4" t="n">
+        <v>1019139</v>
+      </c>
+      <c r="H121" s="4" t="inlineStr">
+        <is>
+          <t>194A for Manisha Kumari: total expenses in books ₹0 is below annual threshold ₹5,000. TDS deduction is voluntary (not wrong if deducted).</t>
+        </is>
+      </c>
+      <c r="I121" s="4" t="inlineStr">
+        <is>
+          <t>TDS was deducted even though aggregate amount is below the threshold. This is not an error — voluntary TDS deduction is valid. No action needed, but note for internal records.</t>
+        </is>
+      </c>
+      <c r="J121" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="4" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" s="4" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="C122" s="4" t="inlineStr">
+        <is>
+          <t>threshold_validation</t>
+        </is>
+      </c>
+      <c r="D122" s="4" t="inlineStr">
+        <is>
+          <t>Suresh Sethia</t>
+        </is>
+      </c>
+      <c r="E122" s="4" t="inlineStr">
+        <is>
+          <t>AAAAA0004A</t>
+        </is>
+      </c>
+      <c r="F122" s="4" t="inlineStr">
+        <is>
+          <t>194A</t>
+        </is>
+      </c>
+      <c r="G122" s="4" t="n">
+        <v>1979192</v>
+      </c>
+      <c r="H122" s="4" t="inlineStr">
+        <is>
+          <t>194A for Suresh Sethia: total expenses in books ₹0 is below annual threshold ₹5,000. TDS deduction is voluntary (not wrong if deducted).</t>
+        </is>
+      </c>
+      <c r="I122" s="4" t="inlineStr">
+        <is>
+          <t>TDS was deducted even though aggregate amount is below the threshold. This is not an error — voluntary TDS deduction is valid. No action needed, but note for internal records.</t>
+        </is>
+      </c>
+      <c r="J122" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="4" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" s="4" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="C123" s="4" t="inlineStr">
+        <is>
+          <t>threshold_validation</t>
+        </is>
+      </c>
+      <c r="D123" s="4" t="inlineStr">
+        <is>
+          <t>Rupa Khaitan</t>
+        </is>
+      </c>
+      <c r="E123" s="4" t="inlineStr">
+        <is>
+          <t>AAAAA0007A</t>
+        </is>
+      </c>
+      <c r="F123" s="4" t="inlineStr">
+        <is>
+          <t>194A</t>
+        </is>
+      </c>
+      <c r="G123" s="4" t="n">
+        <v>81669</v>
+      </c>
+      <c r="H123" s="4" t="inlineStr">
+        <is>
+          <t>194A for Rupa Khaitan: total expenses in books ₹0 is below annual threshold ₹5,000. TDS deduction is voluntary (not wrong if deducted).</t>
+        </is>
+      </c>
+      <c r="I123" s="4" t="inlineStr">
+        <is>
+          <t>TDS was deducted even though aggregate amount is below the threshold. This is not an error — voluntary TDS deduction is valid. No action needed, but note for internal records.</t>
+        </is>
+      </c>
+      <c r="J123" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="4" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" s="4" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="C124" s="4" t="inlineStr">
+        <is>
+          <t>threshold_validation</t>
+        </is>
+      </c>
+      <c r="D124" s="4" t="inlineStr">
+        <is>
+          <t>Akash Nagar</t>
+        </is>
+      </c>
+      <c r="E124" s="4" t="inlineStr">
+        <is>
+          <t>AAAAA0005A</t>
+        </is>
+      </c>
+      <c r="F124" s="4" t="inlineStr">
+        <is>
+          <t>194A</t>
+        </is>
+      </c>
+      <c r="G124" s="4" t="n">
+        <v>1910028</v>
+      </c>
+      <c r="H124" s="4" t="inlineStr">
+        <is>
+          <t>194A for Akash Nagar: total expenses in books ₹0 is below annual threshold ₹5,000. TDS deduction is voluntary (not wrong if deducted).</t>
+        </is>
+      </c>
+      <c r="I124" s="4" t="inlineStr">
+        <is>
+          <t>TDS was deducted even though aggregate amount is below the threshold. This is not an error — voluntary TDS deduction is valid. No action needed, but note for internal records.</t>
+        </is>
+      </c>
+      <c r="J124" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="4" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" s="4" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="C125" s="4" t="inlineStr">
+        <is>
+          <t>threshold_validation</t>
+        </is>
+      </c>
+      <c r="D125" s="4" t="inlineStr">
+        <is>
+          <t>Rahul Shah</t>
+        </is>
+      </c>
+      <c r="E125" s="4" t="inlineStr">
+        <is>
+          <t>AAAAA0006A</t>
+        </is>
+      </c>
+      <c r="F125" s="4" t="inlineStr">
+        <is>
+          <t>194A</t>
+        </is>
+      </c>
+      <c r="G125" s="4" t="n">
+        <v>847707</v>
+      </c>
+      <c r="H125" s="4" t="inlineStr">
+        <is>
+          <t>194A for Rahul Shah: total expenses in books ₹0 is below annual threshold ₹5,000. TDS deduction is voluntary (not wrong if deducted).</t>
+        </is>
+      </c>
+      <c r="I125" s="4" t="inlineStr">
+        <is>
+          <t>TDS was deducted even though aggregate amount is below the threshold. This is not an error — voluntary TDS deduction is valid. No action needed, but note for internal records.</t>
+        </is>
+      </c>
+      <c r="J125" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="4" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" s="4" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="C126" s="4" t="inlineStr">
+        <is>
+          <t>threshold_validation</t>
+        </is>
+      </c>
+      <c r="D126" s="4" t="inlineStr">
+        <is>
+          <t>Karan Kothari</t>
+        </is>
+      </c>
+      <c r="E126" s="4" t="inlineStr">
+        <is>
+          <t>AAAAA0008A</t>
+        </is>
+      </c>
+      <c r="F126" s="4" t="inlineStr">
+        <is>
+          <t>194A</t>
+        </is>
+      </c>
+      <c r="G126" s="4" t="n">
+        <v>596293</v>
+      </c>
+      <c r="H126" s="4" t="inlineStr">
+        <is>
+          <t>194A for Karan Kothari: total expenses in books ₹0 is below annual threshold ₹5,000. TDS deduction is voluntary (not wrong if deducted).</t>
+        </is>
+      </c>
+      <c r="I126" s="4" t="inlineStr">
+        <is>
+          <t>TDS was deducted even though aggregate amount is below the threshold. This is not an error — voluntary TDS deduction is valid. No action needed, but note for internal records.</t>
+        </is>
+      </c>
+      <c r="J126" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="4" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" s="4" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="C127" s="4" t="inlineStr">
+        <is>
+          <t>threshold_validation</t>
+        </is>
+      </c>
+      <c r="D127" s="4" t="inlineStr">
+        <is>
+          <t>Ramesh Lohia</t>
+        </is>
+      </c>
+      <c r="E127" s="4" t="inlineStr">
+        <is>
+          <t>AAAAA0009A</t>
+        </is>
+      </c>
+      <c r="F127" s="4" t="inlineStr">
+        <is>
+          <t>194A</t>
+        </is>
+      </c>
+      <c r="G127" s="4" t="n">
+        <v>311816</v>
+      </c>
+      <c r="H127" s="4" t="inlineStr">
+        <is>
+          <t>194A for Ramesh Lohia: total expenses in books ₹0 is below annual threshold ₹5,000. TDS deduction is voluntary (not wrong if deducted).</t>
+        </is>
+      </c>
+      <c r="I127" s="4" t="inlineStr">
+        <is>
+          <t>TDS was deducted even though aggregate amount is below the threshold. This is not an error — voluntary TDS deduction is valid. No action needed, but note for internal records.</t>
+        </is>
+      </c>
+      <c r="J127" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="4" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" s="4" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="C128" s="4" t="inlineStr">
+        <is>
+          <t>threshold_validation</t>
+        </is>
+      </c>
+      <c r="D128" s="4" t="inlineStr">
+        <is>
+          <t>Raymond Limited</t>
+        </is>
+      </c>
+      <c r="E128" s="4" t="inlineStr">
+        <is>
+          <t>AAACR4896A</t>
+        </is>
+      </c>
+      <c r="F128" s="4" t="inlineStr">
+        <is>
           <t>194Q</t>
         </is>
       </c>
-      <c r="G121" s="4" t="n">
-        <v>381820</v>
-      </c>
-      <c r="H121" s="4" t="inlineStr">
-        <is>
-          <t>194Q for Sai Boutique: Form 26 aggregate ₹381,820 is below annual threshold ₹5,000,000. TDS deduction is voluntary. Note: verify total books expense for this vendor is also below threshold.</t>
-        </is>
-      </c>
-      <c r="I121" s="4" t="inlineStr">
+      <c r="G128" s="4" t="n">
+        <v>1480982</v>
+      </c>
+      <c r="H128" s="4" t="inlineStr">
+        <is>
+          <t>194Q for Raymond Limited: total expenses in books ₹1,480,982 is below annual threshold ₹5,000,000. TDS deduction is voluntary (not wrong if deducted).</t>
+        </is>
+      </c>
+      <c r="I128" s="4" t="inlineStr">
         <is>
           <t>TDS was deducted even though aggregate amount is below the threshold. This is not an error — voluntary TDS deduction is valid. No action needed, but note for internal records.</t>
         </is>
       </c>
-      <c r="J121" s="4" t="inlineStr">
+      <c r="J128" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J121"/>
+  <autoFilter ref="A1:J128"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>